<commit_message>
Add OpenClaw vs Claude Cowork head-to-head comparison tab
New 'OpenClaw vs Claude Cowork' sheet (now the first tab) comparing 35+
attributes across 10 categories:
- Identity & Positioning (category, maturity, open source, use cases)
- Architecture (runtime, execution model, sandboxing, parallel execution)
- Models & Intelligence (model support, context window, quality)
- Compute & Hardware (CPU, RAM, storage, GPU, platform, idle resources, browser)
- Pricing & Cost (license, infra, API, TCO at 3 tiers, hidden costs)
- Extensibility & Integrations (plugins, connectors, MCP, office files)
- Data Sovereignty & Security (data location, security model, compliance)
- Operational Characteristics (always-on, multi-channel, collaboration, setup)
- Performance (task speed, scaling ceiling)
- Summary Verdict (best for, biggest advantage, biggest weakness)

Each row includes a Verdict column highlighting which platform has the edge.

Co-authored-by: ms4674 <ms4674@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/OpenClaw_Architecture_Comparison.xlsx
+++ b/OpenClaw_Architecture_Comparison.xlsx
@@ -7,11 +7,12 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Architecture Comparison" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Compute Requirements" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Pricing Comparison" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Strategic Notes" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="OpenClaw Deep Dive" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="OpenClaw vs Claude Cowork" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Architecture Comparison" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Compute Requirements" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Pricing Comparison" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Strategic Notes" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="OpenClaw Deep Dive" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -21,7 +22,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="4">
+  <fonts count="5">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -44,8 +45,13 @@
       <name val="Calibri"/>
       <sz val="10"/>
     </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <sz val="10"/>
+    </font>
   </fonts>
-  <fills count="6">
+  <fills count="8">
     <fill>
       <patternFill/>
     </fill>
@@ -76,6 +82,18 @@
         <bgColor rgb="00E2EFDA"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E2D9F3"/>
+        <bgColor rgb="00E2D9F3"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FCE4D6"/>
+        <bgColor rgb="00FCE4D6"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -95,15 +113,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -112,7 +127,16 @@
     <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -480,6 +504,1337 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:D53"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="28" customWidth="1" min="1" max="1"/>
+    <col width="44" customWidth="1" min="2" max="2"/>
+    <col width="44" customWidth="1" min="3" max="3"/>
+    <col width="44" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Attribute</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>OpenClaw</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Claude Cowork</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Verdict / Edge</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>— IDENTITY &amp; POSITIONING —</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr"/>
+      <c r="C2" s="2" t="inlineStr"/>
+      <c r="D2" s="2" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>Category</t>
+        </is>
+      </c>
+      <c r="B3" s="4" t="inlineStr">
+        <is>
+          <t>Open-source, self-hosted personal AI assistant.
+General-purpose task automation across
+messaging channels.</t>
+        </is>
+      </c>
+      <c r="C3" s="5" t="inlineStr">
+        <is>
+          <t>Anthropic's desktop AI knowledge-work agent.
+Built into the Claude app for
+macOS (Windows planned).</t>
+        </is>
+      </c>
+      <c r="D3" s="6" t="inlineStr">
+        <is>
+          <t>Both are general-purpose AI assistants (NOT coding agents).
+OpenClaw: messaging-first. Cowork: desktop-first.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>Launch / Maturity</t>
+        </is>
+      </c>
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t>Open-source since 2025.
+68 releases as of March 2026.
+Mature community-driven project.</t>
+        </is>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>Launched Jan 12, 2026 as research preview.
+Built in ~1.5 weeks (by Claude Code itself).
+Still early-stage.</t>
+        </is>
+      </c>
+      <c r="D4" s="6" t="inlineStr">
+        <is>
+          <t>OpenClaw: More mature with larger ecosystem.
+Cowork: Newer but backed by Anthropic.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>Open Source</t>
+        </is>
+      </c>
+      <c r="B5" s="4" t="inlineStr">
+        <is>
+          <t>YES – MIT License.
+322K+ GitHub stars, 62K forks, 360 contributors.</t>
+        </is>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>NO – Proprietary.
+Integrated into Claude app.
+Agent Skills spec is open.</t>
+        </is>
+      </c>
+      <c r="D5" s="6" t="inlineStr">
+        <is>
+          <t>OpenClaw wins for transparency &amp; community.
+Cowork wins for polish &amp; managed experience.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="3" t="inlineStr">
+        <is>
+          <t>Primary Use Cases</t>
+        </is>
+      </c>
+      <c r="B6" s="4" t="inlineStr">
+        <is>
+          <t>Multi-channel messaging automation.
+Email/calendar management.
+Smart home control.
+Workflow automation via cron.
+Browser automation.
+24/7 persistent daemon.</t>
+        </is>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>File management &amp; organization.
+Document processing (XLSX, PPTX, DOCX, PDF).
+Research synthesis &amp; report generation.
+Data extraction (images → spreadsheets).
+Browser automation via Chrome extension.</t>
+        </is>
+      </c>
+      <c r="D6" s="6" t="inlineStr">
+        <is>
+          <t>OpenClaw: Best for persistent, always-on automation across channels.
+Cowork: Best for desktop knowledge work &amp; document tasks.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>— ARCHITECTURE —</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr"/>
+      <c r="C7" s="2" t="inlineStr"/>
+      <c r="D7" s="2" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="3" t="inlineStr">
+        <is>
+          <t>Core Runtime</t>
+        </is>
+      </c>
+      <c r="B8" s="4" t="inlineStr">
+        <is>
+          <t>Node.js long-running daemon (Gateway).
+Message routing, session persistence,
+cron jobs, tool execution.
+Runs 24/7 on user's infrastructure.</t>
+        </is>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>Full Ubuntu 22.04 Linux VM
+running locally on macOS via
+Apple Virtualization.framework.
+Claude Code CLI inside bubblewrap sandbox.</t>
+        </is>
+      </c>
+      <c r="D8" s="6" t="inlineStr">
+        <is>
+          <t>OpenClaw: Lightweight Node.js process.
+Cowork: Heavier (full Linux VM on macOS).
+OpenClaw is more resource-efficient at idle.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="3" t="inlineStr">
+        <is>
+          <t>Execution Model</t>
+        </is>
+      </c>
+      <c r="B9" s="4" t="inlineStr">
+        <is>
+          <t>Gateway-first, channel-native architecture.
+Persistent daemon running 24/7.
+Cron-scheduled autonomous tasks.
+Heartbeat monitoring (15-60 min intervals).</t>
+        </is>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>Session-based desktop agent.
+Runs within Claude app.
+Terminates if computer sleeps.
+No persistent background execution.</t>
+        </is>
+      </c>
+      <c r="D9" s="6" t="inlineStr">
+        <is>
+          <t>OpenClaw: Always-on, autonomous.
+Cowork: Session-dependent, interactive.
+OpenClaw wins for unattended automation.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="3" t="inlineStr">
+        <is>
+          <t>Sandboxing / Isolation</t>
+        </is>
+      </c>
+      <c r="B10" s="4" t="inlineStr">
+        <is>
+          <t>Process-level isolation.
+Docker containers for multi-agent (ClawPod).
+Kubernetes network policies for production.
+Full system access by default.</t>
+        </is>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>VM-level isolation (Apple Virtualization.framework).
+Bubblewrap sandbox + seccomp filtering.
+Folder-specific read/write/create permissions.
+Stronger default isolation.</t>
+        </is>
+      </c>
+      <c r="D10" s="6" t="inlineStr">
+        <is>
+          <t>Cowork: Stronger sandbox by default (VM + seccomp).
+OpenClaw: Full system access (power but risk).
+Cowork wins on security posture.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="3" t="inlineStr">
+        <is>
+          <t>Parallel Execution</t>
+        </is>
+      </c>
+      <c r="B11" s="4" t="inlineStr">
+        <is>
+          <t>Multi-agent via Kubernetes (ClawPod).
+1-100+ agents with per-agent isolation.
+Requires Kubernetes infrastructure.</t>
+        </is>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>Sub-agent coordination.
+Multiple concurrent Claude instances.
+Parallel independent subtasks.
+Native to the app, no infra needed.</t>
+        </is>
+      </c>
+      <c r="D11" s="6" t="inlineStr">
+        <is>
+          <t>Cowork: Easier parallel execution (built-in).
+OpenClaw: More scalable (Kubernetes-based).
+Trade-off: simplicity vs. scale.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>— MODELS &amp; INTELLIGENCE —</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr"/>
+      <c r="C12" s="2" t="inlineStr"/>
+      <c r="D12" s="2" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="3" t="inlineStr">
+        <is>
+          <t>Model Support</t>
+        </is>
+      </c>
+      <c r="B13" s="4" t="inlineStr">
+        <is>
+          <t>Model-agnostic: OpenAI, Anthropic, Google,
+DeepSeek, local models (Ollama, vLLM,
+TensorRT-LLM). Any model via API.</t>
+        </is>
+      </c>
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>Claude family ONLY:
+Claude Opus 4.5/4.6, Sonnet 4.6, Haiku 4.5.
+1M token extended context (Max plans).
+No third-party model support.</t>
+        </is>
+      </c>
+      <c r="D13" s="6" t="inlineStr">
+        <is>
+          <t>OpenClaw: Maximum flexibility (any model).
+Cowork: Locked to Claude (but highest quality).
+OpenClaw wins on choice; Cowork wins on depth.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="3" t="inlineStr">
+        <is>
+          <t>Context Window</t>
+        </is>
+      </c>
+      <c r="B14" s="4" t="inlineStr">
+        <is>
+          <t>Depends on chosen model.
+Typically 128K-200K tokens.
+No built-in extended context.</t>
+        </is>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>Up to 1M tokens (Max plans).
+Extended thinking mode (Max only).
+Progressive disclosure for large files.</t>
+        </is>
+      </c>
+      <c r="D14" s="6" t="inlineStr">
+        <is>
+          <t>Cowork wins: 1M token context + extended thinking
+is significantly larger than typical model defaults.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="3" t="inlineStr">
+        <is>
+          <t>Intelligence Quality</t>
+        </is>
+      </c>
+      <c r="B15" s="4" t="inlineStr">
+        <is>
+          <t>Varies by model selected.
+Can use best-in-class models (Claude Opus)
+or budget models (DeepSeek, Gemini Flash).
+User controls quality-cost trade-off.</t>
+        </is>
+      </c>
+      <c r="C15" s="5" t="inlineStr">
+        <is>
+          <t>Always Claude (Anthropic's top models).
+Consistently high quality.
+No ability to trade down for cost savings.</t>
+        </is>
+      </c>
+      <c r="D15" s="6" t="inlineStr">
+        <is>
+          <t>Cowork: Consistently top-tier quality.
+OpenClaw: Flexible quality (user's choice).
+Different philosophies, not directly comparable.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>— COMPUTE &amp; HARDWARE —</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr"/>
+      <c r="C16" s="2" t="inlineStr"/>
+      <c r="D16" s="2" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="3" t="inlineStr">
+        <is>
+          <t>Minimum CPU</t>
+        </is>
+      </c>
+      <c r="B17" s="4" t="inlineStr">
+        <is>
+          <t>1-2 vCPU</t>
+        </is>
+      </c>
+      <c r="C17" s="5" t="inlineStr">
+        <is>
+          <t>Any modern processor (1-2 cores).
+Recommended: 2+ cores.</t>
+        </is>
+      </c>
+      <c r="D17" s="6" t="inlineStr">
+        <is>
+          <t>Comparable minimum requirements.
+Both lightweight for cloud LLM usage.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="3" t="inlineStr">
+        <is>
+          <t>Minimum RAM</t>
+        </is>
+      </c>
+      <c r="B18" s="4" t="inlineStr">
+        <is>
+          <t>2 GB (hard floor; crashes below).</t>
+        </is>
+      </c>
+      <c r="C18" s="5" t="inlineStr">
+        <is>
+          <t>2 GB minimum; 4-8 GB recommended.
+VM bundle alone consumes significant memory.</t>
+        </is>
+      </c>
+      <c r="D18" s="6" t="inlineStr">
+        <is>
+          <t>Similar floor, but Cowork's VM overhead
+makes 4-8 GB more realistic in practice.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="3" t="inlineStr">
+        <is>
+          <t>Storage</t>
+        </is>
+      </c>
+      <c r="B19" s="4" t="inlineStr">
+        <is>
+          <t>20 GB minimum.
+40-80+ GB recommended.</t>
+        </is>
+      </c>
+      <c r="C19" s="5" t="inlineStr">
+        <is>
+          <t>1 GB installation + 10 GB VM bundle.
+~11 GB minimum; 20+ GB recommended.
+VM image regenerates after sessions.</t>
+        </is>
+      </c>
+      <c r="D19" s="6" t="inlineStr">
+        <is>
+          <t>OpenClaw needs more disk for persistent data.
+Cowork's VM bundle is temporary but large (10 GB).</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="3" t="inlineStr">
+        <is>
+          <t>GPU Required?</t>
+        </is>
+      </c>
+      <c r="B20" s="4" t="inlineStr">
+        <is>
+          <t>NO for cloud LLM.
+YES for local LLM inference.
+(RTX 3060 → A100/H100 depending on model)</t>
+        </is>
+      </c>
+      <c r="C20" s="5" t="inlineStr">
+        <is>
+          <t>NO – cloud inference only.
+No local model support.
+GPU never needed.</t>
+        </is>
+      </c>
+      <c r="D20" s="6" t="inlineStr">
+        <is>
+          <t>OpenClaw: Optional GPU for local models.
+Cowork: No GPU ever needed.
+Cowork simpler; OpenClaw more capable with GPU.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="3" t="inlineStr">
+        <is>
+          <t>Platform Support</t>
+        </is>
+      </c>
+      <c r="B21" s="4" t="inlineStr">
+        <is>
+          <t>Linux, macOS, Windows.
+Docker, Kubernetes, VPS, bare metal.
+Any platform with Node.js.</t>
+        </is>
+      </c>
+      <c r="C21" s="5" t="inlineStr">
+        <is>
+          <t>macOS ONLY (currently).
+Windows support planned.
+Requires Apple Virtualization.framework.</t>
+        </is>
+      </c>
+      <c r="D21" s="6" t="inlineStr">
+        <is>
+          <t>OpenClaw: Runs anywhere.
+Cowork: macOS only (major limitation).
+OpenClaw wins decisively on platform support.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="3" t="inlineStr">
+        <is>
+          <t>Idle Resource Consumption</t>
+        </is>
+      </c>
+      <c r="B22" s="4" t="inlineStr">
+        <is>
+          <t>Node.js Gateway: 300-500 MB RAM, 1-3% CPU.
+Lightweight persistent process.</t>
+        </is>
+      </c>
+      <c r="C22" s="5" t="inlineStr">
+        <is>
+          <t>VM process: reported 24-55% CPU idle on some systems.
+Memory leaks reported over time.
+1.9 GB RAM during VM startup.</t>
+        </is>
+      </c>
+      <c r="D22" s="6" t="inlineStr">
+        <is>
+          <t>OpenClaw: Much lighter at idle (300-500 MB).
+Cowork: Heavier, with reported idle CPU issues.
+OpenClaw wins on resource efficiency.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="3" t="inlineStr">
+        <is>
+          <t>Browser Automation</t>
+        </is>
+      </c>
+      <c r="B23" s="4" t="inlineStr">
+        <is>
+          <t>Playwright-based.
+8 GB RAM hard requirement.
+3 nodes: 75-90% CPU.
+Full browser control.</t>
+        </is>
+      </c>
+      <c r="C23" s="5" t="inlineStr">
+        <is>
+          <t>Chrome extension-based.
+Lighter weight than Playwright.
+Requires Claude for Chrome extension.
+Less programmatic control.</t>
+        </is>
+      </c>
+      <c r="D23" s="6" t="inlineStr">
+        <is>
+          <t>OpenClaw: More powerful (Playwright, full control).
+Cowork: Lighter weight (Chrome extension).
+Trade-off: power vs. simplicity.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>— PRICING &amp; COST —</t>
+        </is>
+      </c>
+      <c r="B24" s="2" t="inlineStr"/>
+      <c r="C24" s="2" t="inlineStr"/>
+      <c r="D24" s="2" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="3" t="inlineStr">
+        <is>
+          <t>Software License</t>
+        </is>
+      </c>
+      <c r="B25" s="4" t="inlineStr">
+        <is>
+          <t>FREE (MIT open source).</t>
+        </is>
+      </c>
+      <c r="C25" s="5" t="inlineStr">
+        <is>
+          <t>Included in Claude subscription:
+Pro: $20/mo | Max 5x: $100/mo |
+Max 20x: $200/mo | Team: $30/user/mo.</t>
+        </is>
+      </c>
+      <c r="D25" s="6" t="inlineStr">
+        <is>
+          <t>OpenClaw: Free software.
+Cowork: $20-200/mo subscription required.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="3" t="inlineStr">
+        <is>
+          <t>Infrastructure Cost</t>
+        </is>
+      </c>
+      <c r="B26" s="4" t="inlineStr">
+        <is>
+          <t>Self-hosted VPS: $4-24/mo.
+Free: Oracle Cloud Always Free.
+User pays hosting.</t>
+        </is>
+      </c>
+      <c r="C26" s="5" t="inlineStr">
+        <is>
+          <t>None – runs on user's Mac.
+No separate infrastructure needed.</t>
+        </is>
+      </c>
+      <c r="D26" s="6" t="inlineStr">
+        <is>
+          <t>OpenClaw: Requires separate hosting ($4-24/mo).
+Cowork: Runs on existing Mac (no extra cost).</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="3" t="inlineStr">
+        <is>
+          <t>LLM / API Cost</t>
+        </is>
+      </c>
+      <c r="B27" s="4" t="inlineStr">
+        <is>
+          <t>Variable: $5-200+/mo.
+Depends on model and usage.
+Cheap models: $5-10/mo.
+Claude Opus heavy: ~$420/mo.</t>
+        </is>
+      </c>
+      <c r="C27" s="5" t="inlineStr">
+        <is>
+          <t>Included in subscription.
+No separate API charges.
+Usage limited by plan tier
+(resets every 5 hours).</t>
+        </is>
+      </c>
+      <c r="D27" s="6" t="inlineStr">
+        <is>
+          <t>OpenClaw: Unbounded variable costs.
+Cowork: Predictable fixed pricing.
+Cowork wins on cost predictability.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="3" t="inlineStr">
+        <is>
+          <t>TCO: Light Use</t>
+        </is>
+      </c>
+      <c r="B28" s="4" t="inlineStr">
+        <is>
+          <t>$10-22/month
+(VPS + budget model APIs).</t>
+        </is>
+      </c>
+      <c r="C28" s="5" t="inlineStr">
+        <is>
+          <t>$20/month (Pro plan).</t>
+        </is>
+      </c>
+      <c r="D28" s="6" t="inlineStr">
+        <is>
+          <t>Comparable at light usage.
+OpenClaw slightly cheaper with budget models.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="3" t="inlineStr">
+        <is>
+          <t>TCO: Moderate Use</t>
+        </is>
+      </c>
+      <c r="B29" s="4" t="inlineStr">
+        <is>
+          <t>$27-72/month
+(VPS + moderate API usage).</t>
+        </is>
+      </c>
+      <c r="C29" s="5" t="inlineStr">
+        <is>
+          <t>$100/month (Max 5x).</t>
+        </is>
+      </c>
+      <c r="D29" s="6" t="inlineStr">
+        <is>
+          <t>OpenClaw cheaper at moderate use.
+Cowork more predictable.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="3" t="inlineStr">
+        <is>
+          <t>TCO: Heavy Use</t>
+        </is>
+      </c>
+      <c r="B30" s="4" t="inlineStr">
+        <is>
+          <t>$62-224+/month per instance.
+Enterprise (100 people): $30-50K/mo.</t>
+        </is>
+      </c>
+      <c r="C30" s="5" t="inlineStr">
+        <is>
+          <t>$200/month (Max 20x).
+Team: $30/user/mo.
+Enterprise: custom.</t>
+        </is>
+      </c>
+      <c r="D30" s="6" t="inlineStr">
+        <is>
+          <t>Cowork cheaper for individual heavy use ($200 flat).
+OpenClaw cheaper at team scale with budget models.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="3" t="inlineStr">
+        <is>
+          <t>Hidden Costs</t>
+        </is>
+      </c>
+      <c r="B31" s="4" t="inlineStr">
+        <is>
+          <t>System prompt token burn: $5-30/mo.
+Heartbeat checks: $0-90/mo.
+Maintenance: 2-5 hrs/mo.
+Model switching overhead.</t>
+        </is>
+      </c>
+      <c r="C31" s="5" t="inlineStr">
+        <is>
+          <t>Cowork sessions burn quota faster
+than regular chat (multi-step reasoning).
+Rate limits reset every 5 hours.
+No overage purchase option.</t>
+        </is>
+      </c>
+      <c r="D31" s="6" t="inlineStr">
+        <is>
+          <t>OpenClaw: Unpredictable API spikes.
+Cowork: Hard rate limits (can't buy more).
+Different risk profiles.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="2" t="inlineStr">
+        <is>
+          <t>— EXTENSIBILITY &amp; INTEGRATIONS —</t>
+        </is>
+      </c>
+      <c r="B32" s="2" t="inlineStr"/>
+      <c r="C32" s="2" t="inlineStr"/>
+      <c r="D32" s="2" t="inlineStr"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="3" t="inlineStr">
+        <is>
+          <t>Plugin / Skill Ecosystem</t>
+        </is>
+      </c>
+      <c r="B33" s="4" t="inlineStr">
+        <is>
+          <t>3,200+ MCP skills on ClawHub.
+Community-built, hot-reloading.
+Cryptographic MCP signing (ECDSA P-256).</t>
+        </is>
+      </c>
+      <c r="C33" s="5" t="inlineStr">
+        <is>
+          <t>11 open-source starter plugins.
+Agent Skills (markdown-based workflow templates).
+Commands (slash-shortcuts).
+Plugins stored locally (org distribution planned).</t>
+        </is>
+      </c>
+      <c r="D33" s="6" t="inlineStr">
+        <is>
+          <t>OpenClaw: Massive existing ecosystem (3,200+).
+Cowork: Early-stage but well-designed.
+OpenClaw wins on ecosystem size today.</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="3" t="inlineStr">
+        <is>
+          <t>Connectors / Integrations</t>
+        </is>
+      </c>
+      <c r="B34" s="4" t="inlineStr">
+        <is>
+          <t>WhatsApp, Telegram, Slack, Discord,
+Signal, iMessage, email, calendar.
+Any MCP server.</t>
+        </is>
+      </c>
+      <c r="C34" s="5" t="inlineStr">
+        <is>
+          <t>37+ native app connectors + Zapier.
+GitHub, Slack, Notion, Google Drive,
+Jira, Salesforce pre-built.
+Most first-party connectors are read-only.</t>
+        </is>
+      </c>
+      <c r="D34" s="6" t="inlineStr">
+        <is>
+          <t>OpenClaw: Messaging-channel focused.
+Cowork: Enterprise SaaS app focused.
+Different integration philosophies.</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="3" t="inlineStr">
+        <is>
+          <t>MCP Support</t>
+        </is>
+      </c>
+      <c r="B35" s="4" t="inlineStr">
+        <is>
+          <t>Full MCP support.
+Every ClawHub skill is an MCP server.
+mcporter CLI for management.
+Hot-reloading, no restart.</t>
+        </is>
+      </c>
+      <c r="C35" s="5" t="inlineStr">
+        <is>
+          <t>Full MCP support.
+Pre-built connectors are MCP-based.
+OAuth authentication flow.
+Connectors maintained by Anthropic + partners.</t>
+        </is>
+      </c>
+      <c r="D35" s="6" t="inlineStr">
+        <is>
+          <t>Both fully MCP-compatible.
+OpenClaw: Community-driven MCP.
+Cowork: Vendor-curated MCP.</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="3" t="inlineStr">
+        <is>
+          <t>Office File Handling</t>
+        </is>
+      </c>
+      <c r="B36" s="4" t="inlineStr">
+        <is>
+          <t>Via community MCP skills.
+Less native office integration.
+Primarily focused on messaging/automation.</t>
+        </is>
+      </c>
+      <c r="C36" s="5" t="inlineStr">
+        <is>
+          <t>Native XLSX, PPTX, DOCX, PDF handling.
+Direct Excel and PowerPoint editing.
+Progressive disclosure for context management.
+Agent Skills spec for office formats.</t>
+        </is>
+      </c>
+      <c r="D36" s="6" t="inlineStr">
+        <is>
+          <t>Cowork wins decisively for document/office work.
+OpenClaw is not designed for file processing.</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="2" t="inlineStr">
+        <is>
+          <t>— DATA SOVEREIGNTY &amp; SECURITY —</t>
+        </is>
+      </c>
+      <c r="B37" s="2" t="inlineStr"/>
+      <c r="C37" s="2" t="inlineStr"/>
+      <c r="D37" s="2" t="inlineStr"/>
+    </row>
+    <row r="38">
+      <c r="A38" s="3" t="inlineStr">
+        <is>
+          <t>Data Location</t>
+        </is>
+      </c>
+      <c r="B38" s="4" t="inlineStr">
+        <is>
+          <t>FULL sovereignty.
+All data stays on user's infrastructure.
+No data sent to third parties
+(except chosen LLM API calls).</t>
+        </is>
+      </c>
+      <c r="C38" s="5" t="inlineStr">
+        <is>
+          <t>Partial sovereignty.
+Files processed locally in VM.
+Prompts/responses go to Anthropic's cloud.
+Team/Enterprise: not used for training.</t>
+        </is>
+      </c>
+      <c r="D38" s="6" t="inlineStr">
+        <is>
+          <t>OpenClaw: Full data control.
+Cowork: Files local, but prompts go to Anthropic.
+OpenClaw wins for data sovereignty.</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="3" t="inlineStr">
+        <is>
+          <t>Security Model</t>
+        </is>
+      </c>
+      <c r="B39" s="4" t="inlineStr">
+        <is>
+          <t>Full system access by default.
+User configures restrictions.
+Network policies via Kubernetes.
+Cryptographic MCP signing.</t>
+        </is>
+      </c>
+      <c r="C39" s="5" t="inlineStr">
+        <is>
+          <t>VM sandbox + bubblewrap + seccomp.
+Folder-specific permissions (read/write/create).
+Explicit directory approval required.
+KNOWN: Prompt injection vulnerability
+(file exfiltration via whitelisted APIs, unpatched Jan 2026).</t>
+        </is>
+      </c>
+      <c r="D39" s="6" t="inlineStr">
+        <is>
+          <t>Cowork: Better default sandboxing.
+OpenClaw: Better production security (K8s).
+Cowork has known unpatched vulnerability.</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="3" t="inlineStr">
+        <is>
+          <t>Enterprise Compliance</t>
+        </is>
+      </c>
+      <c r="B40" s="4" t="inlineStr">
+        <is>
+          <t>No built-in compliance features.
+User implements own controls.
+No SSO/SCIM/audit logs natively.</t>
+        </is>
+      </c>
+      <c r="C40" s="5" t="inlineStr">
+        <is>
+          <t>SSO/SCIM (Enterprise plan).
+Audit logs planned.
+Connector-level access controls.
+Service account support.</t>
+        </is>
+      </c>
+      <c r="D40" s="6" t="inlineStr">
+        <is>
+          <t>Cowork: Better enterprise compliance features.
+OpenClaw: Requires DIY compliance setup.</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="2" t="inlineStr">
+        <is>
+          <t>— OPERATIONAL CHARACTERISTICS —</t>
+        </is>
+      </c>
+      <c r="B41" s="2" t="inlineStr"/>
+      <c r="C41" s="2" t="inlineStr"/>
+      <c r="D41" s="2" t="inlineStr"/>
+    </row>
+    <row r="42">
+      <c r="A42" s="3" t="inlineStr">
+        <is>
+          <t>Always-On Availability</t>
+        </is>
+      </c>
+      <c r="B42" s="4" t="inlineStr">
+        <is>
+          <t>YES – runs as persistent daemon 24/7.
+Cron-scheduled autonomous tasks.
+Heartbeat monitoring.
+Survives user disconnection.</t>
+        </is>
+      </c>
+      <c r="C42" s="5" t="inlineStr">
+        <is>
+          <t>NO – session-based.
+Terminates if computer sleeps.
+Requires active Mac session.
+No background persistence.</t>
+        </is>
+      </c>
+      <c r="D42" s="6" t="inlineStr">
+        <is>
+          <t>OpenClaw wins decisively.
+Always-on is OpenClaw's core strength.
+Cowork requires active desktop session.</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="3" t="inlineStr">
+        <is>
+          <t>Multi-Channel Communication</t>
+        </is>
+      </c>
+      <c r="B43" s="4" t="inlineStr">
+        <is>
+          <t>Native multi-channel:
+WhatsApp, Telegram, Slack, Discord,
+Signal, iMessage simultaneously.
+Channel-agnostic agent.</t>
+        </is>
+      </c>
+      <c r="C43" s="5" t="inlineStr">
+        <is>
+          <t>Single interface (Claude app).
+Connectors for reading from external apps.
+No native messaging channel support.</t>
+        </is>
+      </c>
+      <c r="D43" s="6" t="inlineStr">
+        <is>
+          <t>OpenClaw wins decisively.
+Multi-channel messaging is its raison d'être.
+Cowork is desktop-app only.</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="3" t="inlineStr">
+        <is>
+          <t>Collaboration Features</t>
+        </is>
+      </c>
+      <c r="B44" s="4" t="inlineStr">
+        <is>
+          <t>Multi-agent coordination.
+Hierarchical agent patterns.
+Shared workspace via Kubernetes.</t>
+        </is>
+      </c>
+      <c r="C44" s="5" t="inlineStr">
+        <is>
+          <t>No sharing or collaboration features.
+Single-user desktop experience.
+Team distribution planned (future).</t>
+        </is>
+      </c>
+      <c r="D44" s="6" t="inlineStr">
+        <is>
+          <t>OpenClaw: Better for team/multi-agent use.
+Cowork: Single-user only (for now).</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="3" t="inlineStr">
+        <is>
+          <t>Setup Complexity</t>
+        </is>
+      </c>
+      <c r="B45" s="4" t="inlineStr">
+        <is>
+          <t>Moderate-High.
+Requires VPS provisioning, Docker/K8s,
+API key configuration, channel setup.
+2-5 hrs/mo maintenance.</t>
+        </is>
+      </c>
+      <c r="C45" s="5" t="inlineStr">
+        <is>
+          <t>Low.
+Built into Claude app.
+One-click folder permissions.
+No infrastructure to manage.</t>
+        </is>
+      </c>
+      <c r="D45" s="6" t="inlineStr">
+        <is>
+          <t>Cowork wins on ease of setup.
+OpenClaw requires technical expertise.
+Cowork: minutes to start. OpenClaw: hours.</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="3" t="inlineStr">
+        <is>
+          <t>Maintenance Burden</t>
+        </is>
+      </c>
+      <c r="B46" s="4" t="inlineStr">
+        <is>
+          <t>2-5 hours/month.
+Updates, troubleshooting, config.
+API key rotation, model switching.
+Infra monitoring.</t>
+        </is>
+      </c>
+      <c r="C46" s="5" t="inlineStr">
+        <is>
+          <t>Zero maintenance.
+Managed by Anthropic.
+Automatic updates via Claude app.</t>
+        </is>
+      </c>
+      <c r="D46" s="6" t="inlineStr">
+        <is>
+          <t>Cowork wins: zero maintenance.
+OpenClaw: ongoing operational overhead.</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="2" t="inlineStr">
+        <is>
+          <t>— PERFORMANCE —</t>
+        </is>
+      </c>
+      <c r="B47" s="2" t="inlineStr"/>
+      <c r="C47" s="2" t="inlineStr"/>
+      <c r="D47" s="2" t="inlineStr"/>
+    </row>
+    <row r="48">
+      <c r="A48" s="3" t="inlineStr">
+        <is>
+          <t>Task Completion Speed</t>
+        </is>
+      </c>
+      <c r="B48" s="4" t="inlineStr">
+        <is>
+          <t>Depends on chosen model and infrastructure.
+No published benchmarks.
+Variable based on API latency.</t>
+        </is>
+      </c>
+      <c r="C48" s="5" t="inlineStr">
+        <is>
+          <t>92% reduction in task time vs. manual work
+(3.1 hrs → ~15 min, per Anthropic data).
+Parallel execution reduces multi-task time
+to duration of longest single task.</t>
+        </is>
+      </c>
+      <c r="D48" s="6" t="inlineStr">
+        <is>
+          <t>Cowork: Published performance data.
+OpenClaw: No comparable benchmarks.
+Cowork has better documented productivity gains.</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="3" t="inlineStr">
+        <is>
+          <t>Scaling Ceiling</t>
+        </is>
+      </c>
+      <c r="B49" s="4" t="inlineStr">
+        <is>
+          <t>Kubernetes: 1 to 100+ agents.
+Per-agent resource isolation.
+Network policies.
+Production-grade multi-tenancy.</t>
+        </is>
+      </c>
+      <c r="C49" s="5" t="inlineStr">
+        <is>
+          <t>Single Mac desktop.
+Multiple conversations share one VM.
+No horizontal scaling.
+Capped by Mac hardware.</t>
+        </is>
+      </c>
+      <c r="D49" s="6" t="inlineStr">
+        <is>
+          <t>OpenClaw wins on scaling.
+Cowork is fundamentally single-machine.
+OpenClaw designed for enterprise scale.</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="2" t="inlineStr">
+        <is>
+          <t>— SUMMARY VERDICT —</t>
+        </is>
+      </c>
+      <c r="B50" s="2" t="inlineStr"/>
+      <c r="C50" s="2" t="inlineStr"/>
+      <c r="D50" s="2" t="inlineStr"/>
+    </row>
+    <row r="51">
+      <c r="A51" s="3" t="inlineStr">
+        <is>
+          <t>Best For</t>
+        </is>
+      </c>
+      <c r="B51" s="4" t="inlineStr">
+        <is>
+          <t>Always-on automation.
+Multi-channel messaging agents.
+Privacy-first deployments.
+Budget-conscious users.
+Teams wanting full control.</t>
+        </is>
+      </c>
+      <c r="C51" s="5" t="inlineStr">
+        <is>
+          <t>Desktop knowledge work.
+Document processing &amp; organization.
+Polished single-user experience.
+Users wanting zero-maintenance.
+macOS-native workflows.</t>
+        </is>
+      </c>
+      <c r="D51" s="6" t="inlineStr">
+        <is>
+          <t>NOT direct competitors.
+OpenClaw = persistent messaging automation platform.
+Cowork = desktop productivity agent.
+Complementary tools for different workflows.</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="3" t="inlineStr">
+        <is>
+          <t>Biggest Advantage</t>
+        </is>
+      </c>
+      <c r="B52" s="4" t="inlineStr">
+        <is>
+          <t>Open source, model-agnostic,
+always-on, full data sovereignty,
+massive plugin ecosystem,
+lowest possible TCO.</t>
+        </is>
+      </c>
+      <c r="C52" s="5" t="inlineStr">
+        <is>
+          <t>Zero setup, polished UX,
+enterprise-grade Claude models,
+strong sandboxing,
+predictable fixed pricing,
+native document handling.</t>
+        </is>
+      </c>
+      <c r="D52" s="6" t="inlineStr">
+        <is>
+          <t>OpenClaw: Control &amp; flexibility.
+Cowork: Simplicity &amp; polish.</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="3" t="inlineStr">
+        <is>
+          <t>Biggest Weakness</t>
+        </is>
+      </c>
+      <c r="B53" s="4" t="inlineStr">
+        <is>
+          <t>Operational overhead.
+Self-hosting maintenance burden.
+Not designed for document/office work.
+No native enterprise compliance.</t>
+        </is>
+      </c>
+      <c r="C53" s="5" t="inlineStr">
+        <is>
+          <t>macOS only.
+Session-dependent (no 24/7 operation).
+Claude-only (vendor lock-in).
+Known security vulnerability.
+No multi-channel messaging.</t>
+        </is>
+      </c>
+      <c r="D53" s="6" t="inlineStr">
+        <is>
+          <t>OpenClaw: Complexity.
+Cowork: Limited platform &amp; model choice.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:K10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -554,182 +1909,182 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="inlineStr">
+      <c r="A2" s="7" t="inlineStr">
         <is>
           <t>Category</t>
         </is>
       </c>
-      <c r="B2" s="3" t="inlineStr">
+      <c r="B2" s="8" t="inlineStr">
         <is>
           <t>General-purpose AI assistant</t>
         </is>
       </c>
-      <c r="C2" s="2" t="inlineStr">
+      <c r="C2" s="7" t="inlineStr">
         <is>
           <t>Autonomous SW engineer</t>
         </is>
       </c>
-      <c r="D2" s="2" t="inlineStr">
+      <c r="D2" s="7" t="inlineStr">
         <is>
           <t>AI-native IDE</t>
         </is>
       </c>
-      <c r="E2" s="2" t="inlineStr">
+      <c r="E2" s="7" t="inlineStr">
         <is>
           <t>IDE-integrated copilot</t>
         </is>
       </c>
-      <c r="F2" s="2" t="inlineStr">
+      <c r="F2" s="7" t="inlineStr">
         <is>
           <t>Terminal-native agent</t>
         </is>
       </c>
-      <c r="G2" s="2" t="inlineStr">
+      <c r="G2" s="7" t="inlineStr">
         <is>
           <t>Agentic IDE</t>
         </is>
       </c>
-      <c r="H2" s="2" t="inlineStr">
+      <c r="H2" s="7" t="inlineStr">
         <is>
           <t>Autonomous coding agent</t>
         </is>
       </c>
-      <c r="I2" s="2" t="inlineStr">
+      <c r="I2" s="7" t="inlineStr">
         <is>
           <t>Autonomous app builder</t>
         </is>
       </c>
-      <c r="J2" s="2" t="inlineStr">
+      <c r="J2" s="7" t="inlineStr">
         <is>
           <t>AWS-native coding agent</t>
         </is>
       </c>
-      <c r="K2" s="2" t="inlineStr">
+      <c r="K2" s="7" t="inlineStr">
         <is>
           <t>Open-source coding agent</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="2" t="inlineStr">
+      <c r="A3" s="7" t="inlineStr">
         <is>
           <t>Open Source</t>
         </is>
       </c>
-      <c r="B3" s="3" t="inlineStr">
+      <c r="B3" s="8" t="inlineStr">
         <is>
           <t>Yes – MIT License
 322K+ GitHub stars</t>
         </is>
       </c>
-      <c r="C3" s="2" t="inlineStr">
+      <c r="C3" s="7" t="inlineStr">
         <is>
           <t>No – Proprietary</t>
         </is>
       </c>
-      <c r="D3" s="2" t="inlineStr">
+      <c r="D3" s="7" t="inlineStr">
         <is>
           <t>No – Proprietary
 (Composer model details shared)</t>
         </is>
       </c>
-      <c r="E3" s="2" t="inlineStr">
+      <c r="E3" s="7" t="inlineStr">
         <is>
           <t>No – Proprietary</t>
         </is>
       </c>
-      <c r="F3" s="2" t="inlineStr">
+      <c r="F3" s="7" t="inlineStr">
         <is>
           <t>No – Proprietary</t>
         </is>
       </c>
-      <c r="G3" s="2" t="inlineStr">
+      <c r="G3" s="7" t="inlineStr">
         <is>
           <t>No – Proprietary</t>
         </is>
       </c>
-      <c r="H3" s="2" t="inlineStr">
+      <c r="H3" s="7" t="inlineStr">
         <is>
           <t>No – Proprietary</t>
         </is>
       </c>
-      <c r="I3" s="2" t="inlineStr">
+      <c r="I3" s="7" t="inlineStr">
         <is>
           <t>No – Proprietary</t>
         </is>
       </c>
-      <c r="J3" s="2" t="inlineStr">
+      <c r="J3" s="7" t="inlineStr">
         <is>
           <t>No – Proprietary</t>
         </is>
       </c>
-      <c r="K3" s="2" t="inlineStr">
+      <c r="K3" s="7" t="inlineStr">
         <is>
           <t>Yes – MIT License</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="4" t="inlineStr">
+      <c r="A4" s="3" t="inlineStr">
         <is>
           <t>Primary Language / Stack</t>
         </is>
       </c>
-      <c r="B4" s="5" t="inlineStr">
+      <c r="B4" s="4" t="inlineStr">
         <is>
           <t>TypeScript (87.8%)
 Node.js runtime</t>
         </is>
       </c>
-      <c r="C4" s="4" t="inlineStr">
+      <c r="C4" s="3" t="inlineStr">
         <is>
           <t>Compound AI system
 Multiple specialized models</t>
         </is>
       </c>
-      <c r="D4" s="4" t="inlineStr">
+      <c r="D4" s="3" t="inlineStr">
         <is>
           <t>Electron (VS Code fork)
 Custom MoE model (Composer)</t>
         </is>
       </c>
-      <c r="E4" s="4" t="inlineStr">
+      <c r="E4" s="3" t="inlineStr">
         <is>
           <t>Cloud-hosted
 Multiple LLM backends</t>
         </is>
       </c>
-      <c r="F4" s="4" t="inlineStr">
+      <c r="F4" s="3" t="inlineStr">
         <is>
           <t>Cloud-hosted
 Claude model family</t>
         </is>
       </c>
-      <c r="G4" s="4" t="inlineStr">
+      <c r="G4" s="3" t="inlineStr">
         <is>
           <t>Electron (VS Code fork)
 SWE-1.5 proprietary model</t>
         </is>
       </c>
-      <c r="H4" s="4" t="inlineStr">
+      <c r="H4" s="3" t="inlineStr">
         <is>
           <t>Cloud-hosted
 Multi-model sampling</t>
         </is>
       </c>
-      <c r="I4" s="4" t="inlineStr">
+      <c r="I4" s="3" t="inlineStr">
         <is>
           <t>Cloud-hosted
 Claude Sonnet 4 + GPT-4o</t>
         </is>
       </c>
-      <c r="J4" s="4" t="inlineStr">
+      <c r="J4" s="3" t="inlineStr">
         <is>
           <t>Cloud-hosted
 Claude models</t>
         </is>
       </c>
-      <c r="K4" s="4" t="inlineStr">
+      <c r="K4" s="3" t="inlineStr">
         <is>
           <t>Python
 YAML-config driven</t>
@@ -737,12 +2092,12 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="2" t="inlineStr">
+      <c r="A5" s="7" t="inlineStr">
         <is>
           <t>Core Architecture</t>
         </is>
       </c>
-      <c r="B5" s="3" t="inlineStr">
+      <c r="B5" s="8" t="inlineStr">
         <is>
           <t>Long-running Node.js daemon (Gateway).
 Message routing, session persistence,
@@ -751,7 +2106,7 @@
 CPU-bound for tool/browser execution.</t>
         </is>
       </c>
-      <c r="C5" s="2" t="inlineStr">
+      <c r="C5" s="7" t="inlineStr">
         <is>
           <t>Compound AI system:
 - Planner (high-reasoning model)
@@ -761,7 +2116,7 @@
 Separates planning from execution.</t>
         </is>
       </c>
-      <c r="D5" s="2" t="inlineStr">
+      <c r="D5" s="7" t="inlineStr">
         <is>
           <t>ReAct loop with context injection.
 MoE model (Composer) trained via RL.
@@ -769,7 +2124,7 @@
 Sandboxed file/network access.</t>
         </is>
       </c>
-      <c r="E5" s="2" t="inlineStr">
+      <c r="E5" s="7" t="inlineStr">
         <is>
           <t>Cloud-hosted inference.
 GitHub Issues → PR generation.
@@ -777,7 +2132,7 @@
 Deep GitHub ecosystem integration.</t>
         </is>
       </c>
-      <c r="F5" s="2" t="inlineStr">
+      <c r="F5" s="7" t="inlineStr">
         <is>
           <t>Terminal-native autonomous agent.
 Cloud inference only.
@@ -785,7 +2140,7 @@
 API or subscription billing.</t>
         </is>
       </c>
-      <c r="G5" s="2" t="inlineStr">
+      <c r="G5" s="7" t="inlineStr">
         <is>
           <t>Cascade agent with hybrid indexing
 (AST + semantic embeddings).
@@ -794,7 +2149,7 @@
 21 MCP connectors.</t>
         </is>
       </c>
-      <c r="H5" s="2" t="inlineStr">
+      <c r="H5" s="7" t="inlineStr">
         <is>
           <t>HyperCode codebase representation.
 ByteRank retrieval.
@@ -802,7 +2157,7 @@
 Multi-model task-dependent sampling.</t>
         </is>
       </c>
-      <c r="I5" s="2" t="inlineStr">
+      <c r="I5" s="7" t="inlineStr">
         <is>
           <t>Full-stack autonomous builder.
 Parallel task execution.
@@ -810,7 +2165,7 @@
 One-click deployment.</t>
         </is>
       </c>
-      <c r="J5" s="2" t="inlineStr">
+      <c r="J5" s="7" t="inlineStr">
         <is>
           <t>IDE + CLI + workspace agent.
 AWS API integration.
@@ -818,7 +2173,7 @@
 Architecture diagram generation.</t>
         </is>
       </c>
-      <c r="K5" s="2" t="inlineStr">
+      <c r="K5" s="7" t="inlineStr">
         <is>
           <t>YAML-config agent framework.
 SWE-ReX remote execution.
@@ -828,19 +2183,19 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="4" t="inlineStr">
+      <c r="A6" s="3" t="inlineStr">
         <is>
           <t>Deployment Model</t>
         </is>
       </c>
-      <c r="B6" s="5" t="inlineStr">
+      <c r="B6" s="4" t="inlineStr">
         <is>
           <t>Self-hosted (VPS, bare metal,
 Kubernetes, Docker).
 Full data sovereignty.</t>
         </is>
       </c>
-      <c r="C6" s="4" t="inlineStr">
+      <c r="C6" s="3" t="inlineStr">
         <is>
           <t>SaaS (multi-tenant) or
 Customer-dedicated SaaS
@@ -848,49 +2203,49 @@
 AWS PrivateLink / IPSec.</t>
         </is>
       </c>
-      <c r="D6" s="4" t="inlineStr">
+      <c r="D6" s="3" t="inlineStr">
         <is>
           <t>Desktop app (local IDE).
 Cloud agents for background tasks.</t>
         </is>
       </c>
-      <c r="E6" s="4" t="inlineStr">
+      <c r="E6" s="3" t="inlineStr">
         <is>
           <t>Cloud SaaS.
 GitHub-native integration.</t>
         </is>
       </c>
-      <c r="F6" s="4" t="inlineStr">
+      <c r="F6" s="3" t="inlineStr">
         <is>
           <t>Cloud SaaS.
 No self-hosting option.</t>
         </is>
       </c>
-      <c r="G6" s="4" t="inlineStr">
+      <c r="G6" s="3" t="inlineStr">
         <is>
           <t>Desktop app (local IDE).
 Cloud inference.</t>
         </is>
       </c>
-      <c r="H6" s="4" t="inlineStr">
+      <c r="H6" s="3" t="inlineStr">
         <is>
           <t>Cloud SaaS.
 Platform-managed or BYOM compute.</t>
         </is>
       </c>
-      <c r="I6" s="4" t="inlineStr">
+      <c r="I6" s="3" t="inlineStr">
         <is>
           <t>Cloud SaaS.
 Replit-hosted infrastructure.</t>
         </is>
       </c>
-      <c r="J6" s="4" t="inlineStr">
+      <c r="J6" s="3" t="inlineStr">
         <is>
           <t>Cloud SaaS.
 AWS-native deployment.</t>
         </is>
       </c>
-      <c r="K6" s="4" t="inlineStr">
+      <c r="K6" s="3" t="inlineStr">
         <is>
           <t>Self-hosted.
 Local Docker, AWS, Modal,
@@ -899,67 +2254,67 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="4" t="inlineStr">
+      <c r="A7" s="3" t="inlineStr">
         <is>
           <t>Model Support</t>
         </is>
       </c>
-      <c r="B7" s="5" t="inlineStr">
+      <c r="B7" s="4" t="inlineStr">
         <is>
           <t>Any model: OpenAI, Anthropic,
 Google, local (Ollama, vLLM,
 TensorRT-LLM). Model-agnostic.</t>
         </is>
       </c>
-      <c r="C7" s="4" t="inlineStr">
+      <c r="C7" s="3" t="inlineStr">
         <is>
           <t>Proprietary compound models.
 No user model choice.</t>
         </is>
       </c>
-      <c r="D7" s="4" t="inlineStr">
+      <c r="D7" s="3" t="inlineStr">
         <is>
           <t>Custom Composer MoE +
 Claude, GPT-4, Gemini access.</t>
         </is>
       </c>
-      <c r="E7" s="4" t="inlineStr">
+      <c r="E7" s="3" t="inlineStr">
         <is>
           <t>Multiple LLM backends
 (model selection per request).</t>
         </is>
       </c>
-      <c r="F7" s="4" t="inlineStr">
+      <c r="F7" s="3" t="inlineStr">
         <is>
           <t>Claude family only
 (Opus 4.6, Sonnet 4.6, Haiku 4.5).</t>
         </is>
       </c>
-      <c r="G7" s="4" t="inlineStr">
+      <c r="G7" s="3" t="inlineStr">
         <is>
           <t>Proprietary SWE-1.5 +
 third-party model access.</t>
         </is>
       </c>
-      <c r="H7" s="4" t="inlineStr">
+      <c r="H7" s="3" t="inlineStr">
         <is>
           <t>Multi-model with task-dependent
 selection and multipliers.</t>
         </is>
       </c>
-      <c r="I7" s="4" t="inlineStr">
+      <c r="I7" s="3" t="inlineStr">
         <is>
           <t>Claude Sonnet 4 + GPT-4o.
 No user model choice.</t>
         </is>
       </c>
-      <c r="J7" s="4" t="inlineStr">
+      <c r="J7" s="3" t="inlineStr">
         <is>
           <t>Claude models.
 No user model choice.</t>
         </is>
       </c>
-      <c r="K7" s="4" t="inlineStr">
+      <c r="K7" s="3" t="inlineStr">
         <is>
           <t>Any model: GPT-4o, Claude,
 local models. Fully configurable.</t>
@@ -967,12 +2322,12 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="4" t="inlineStr">
+      <c r="A8" s="3" t="inlineStr">
         <is>
           <t>Agent Paradigm</t>
         </is>
       </c>
-      <c r="B8" s="5" t="inlineStr">
+      <c r="B8" s="4" t="inlineStr">
         <is>
           <t>Persistent daemon.
 Multi-channel messaging.
@@ -980,63 +2335,63 @@
 Browser automation.</t>
         </is>
       </c>
-      <c r="C8" s="4" t="inlineStr">
+      <c r="C8" s="3" t="inlineStr">
         <is>
           <t>Fully autonomous loop.
 Own environment (Devbox).
 Planner-Critic-Coder pipeline.</t>
         </is>
       </c>
-      <c r="D8" s="4" t="inlineStr">
+      <c r="D8" s="3" t="inlineStr">
         <is>
           <t>Interactive agent in IDE.
 Sub-agent spawning.
 Background cloud agents.</t>
         </is>
       </c>
-      <c r="E8" s="4" t="inlineStr">
+      <c r="E8" s="3" t="inlineStr">
         <is>
           <t>Task-centric (Issue → PR).
 Inline suggestions.
 Chat-based assistance.</t>
         </is>
       </c>
-      <c r="F8" s="4" t="inlineStr">
+      <c r="F8" s="3" t="inlineStr">
         <is>
           <t>Terminal-based autonomous agent.
 ReAct loop.
 File/shell access.</t>
         </is>
       </c>
-      <c r="G8" s="4" t="inlineStr">
+      <c r="G8" s="3" t="inlineStr">
         <is>
           <t>Cascade planner.
 Multi-file reasoning.
 Flow-aware context tracking.</t>
         </is>
       </c>
-      <c r="H8" s="4" t="inlineStr">
+      <c r="H8" s="3" t="inlineStr">
         <is>
           <t>Autonomous task execution.
 Custom subagent delegation.
 CI/CD integration.</t>
         </is>
       </c>
-      <c r="I8" s="4" t="inlineStr">
+      <c r="I8" s="3" t="inlineStr">
         <is>
           <t>Autonomous build loop.
 Iterative debugging.
 Deploy-in-loop.</t>
         </is>
       </c>
-      <c r="J8" s="4" t="inlineStr">
+      <c r="J8" s="3" t="inlineStr">
         <is>
           <t>Agentic requests.
 Code transformation.
 AWS service integration.</t>
         </is>
       </c>
-      <c r="K8" s="4" t="inlineStr">
+      <c r="K8" s="3" t="inlineStr">
         <is>
           <t>Autonomous fix loop.
 GitHub issue resolution.
@@ -1045,71 +2400,71 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="4" t="inlineStr">
+      <c r="A9" s="3" t="inlineStr">
         <is>
           <t>Extensibility / Plugins</t>
         </is>
       </c>
-      <c r="B9" s="5" t="inlineStr">
+      <c r="B9" s="4" t="inlineStr">
         <is>
           <t>3,200+ MCP skills on ClawHub.
 Hot-reloading plugins.
 Cryptographic MCP signing.</t>
         </is>
       </c>
-      <c r="C9" s="4" t="inlineStr">
+      <c r="C9" s="3" t="inlineStr">
         <is>
           <t>Limited – Slack, IDE extensions.
 No plugin marketplace.</t>
         </is>
       </c>
-      <c r="D9" s="4" t="inlineStr">
+      <c r="D9" s="3" t="inlineStr">
         <is>
           <t>MCP support.
 Custom rules/commands.
 Extensions via VS Code ecosystem.</t>
         </is>
       </c>
-      <c r="E9" s="4" t="inlineStr">
+      <c r="E9" s="3" t="inlineStr">
         <is>
           <t>GitHub Actions integration.
 Limited extension model.</t>
         </is>
       </c>
-      <c r="F9" s="4" t="inlineStr">
+      <c r="F9" s="3" t="inlineStr">
         <is>
           <t>MCP support.
 Bash tool access.</t>
         </is>
       </c>
-      <c r="G9" s="4" t="inlineStr">
+      <c r="G9" s="3" t="inlineStr">
         <is>
           <t>21 first-party MCP connectors
 (Figma, Slack, Stripe, etc.).
 40+ IDE compatibility bridges.</t>
         </is>
       </c>
-      <c r="H9" s="4" t="inlineStr">
+      <c r="H9" s="3" t="inlineStr">
         <is>
           <t>Custom Droids (subagents).
 Linter/analyzer integration.</t>
         </is>
       </c>
-      <c r="I9" s="4" t="inlineStr">
+      <c r="I9" s="3" t="inlineStr">
         <is>
           <t>Figma import.
 Database integrations.
 Deployment pipelines.</t>
         </is>
       </c>
-      <c r="J9" s="4" t="inlineStr">
+      <c r="J9" s="3" t="inlineStr">
         <is>
           <t>AWS service integrations.
 IDE plugins (VS Code, JetBrains,
 Visual Studio, Eclipse).</t>
         </is>
       </c>
-      <c r="K9" s="4" t="inlineStr">
+      <c r="K9" s="3" t="inlineStr">
         <is>
           <t>YAML-based configuration.
 Custom tool definitions.
@@ -1118,58 +2473,58 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="2" t="inlineStr">
+      <c r="A10" s="7" t="inlineStr">
         <is>
           <t>SWE-bench Verified Score</t>
         </is>
       </c>
-      <c r="B10" s="3" t="inlineStr">
+      <c r="B10" s="8" t="inlineStr">
         <is>
           <t>N/A (not a coding agent)</t>
         </is>
       </c>
-      <c r="C10" s="2" t="inlineStr">
+      <c r="C10" s="7" t="inlineStr">
         <is>
           <t>~55-60% (estimated)</t>
         </is>
       </c>
-      <c r="D10" s="2" t="inlineStr">
+      <c r="D10" s="7" t="inlineStr">
         <is>
           <t>Not publicly disclosed</t>
         </is>
       </c>
-      <c r="E10" s="2" t="inlineStr">
+      <c r="E10" s="7" t="inlineStr">
         <is>
           <t>Not publicly disclosed</t>
         </is>
       </c>
-      <c r="F10" s="2" t="inlineStr">
+      <c r="F10" s="7" t="inlineStr">
         <is>
           <t>79.6-82%
 (highest as of early 2026)</t>
         </is>
       </c>
-      <c r="G10" s="2" t="inlineStr">
+      <c r="G10" s="7" t="inlineStr">
         <is>
           <t>Not publicly disclosed</t>
         </is>
       </c>
-      <c r="H10" s="2" t="inlineStr">
+      <c r="H10" s="7" t="inlineStr">
         <is>
           <t>Not publicly disclosed</t>
         </is>
       </c>
-      <c r="I10" s="2" t="inlineStr">
+      <c r="I10" s="7" t="inlineStr">
         <is>
           <t>Not publicly disclosed</t>
         </is>
       </c>
-      <c r="J10" s="2" t="inlineStr">
+      <c r="J10" s="7" t="inlineStr">
         <is>
           <t>Not publicly disclosed</t>
         </is>
       </c>
-      <c r="K10" s="2" t="inlineStr">
+      <c r="K10" s="7" t="inlineStr">
         <is>
           <t>~65% (mini-swe-agent)</t>
         </is>
@@ -1180,7 +2535,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1235,47 +2590,47 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="6" t="inlineStr">
+      <c r="A2" s="2" t="inlineStr">
         <is>
           <t>— MINIMUM HARDWARE —</t>
         </is>
       </c>
-      <c r="B2" s="6" t="inlineStr"/>
-      <c r="C2" s="6" t="inlineStr"/>
-      <c r="D2" s="6" t="inlineStr"/>
-      <c r="E2" s="6" t="inlineStr"/>
-      <c r="F2" s="6" t="inlineStr"/>
+      <c r="B2" s="2" t="inlineStr"/>
+      <c r="C2" s="2" t="inlineStr"/>
+      <c r="D2" s="2" t="inlineStr"/>
+      <c r="E2" s="2" t="inlineStr"/>
+      <c r="F2" s="2" t="inlineStr"/>
     </row>
     <row r="3">
-      <c r="A3" s="4" t="inlineStr">
+      <c r="A3" s="3" t="inlineStr">
         <is>
           <t>CPU (Minimum)</t>
         </is>
       </c>
-      <c r="B3" s="5" t="inlineStr">
+      <c r="B3" s="4" t="inlineStr">
         <is>
           <t>1-2 vCPU</t>
         </is>
       </c>
-      <c r="C3" s="4" t="inlineStr">
+      <c r="C3" s="3" t="inlineStr">
         <is>
           <t>70+ vCPUs (AWS VPC)
 i3.metal instances</t>
         </is>
       </c>
-      <c r="D3" s="4" t="inlineStr">
+      <c r="D3" s="3" t="inlineStr">
         <is>
           <t>N/A (cloud-hosted;
 user runs desktop IDE)</t>
         </is>
       </c>
-      <c r="E3" s="4" t="inlineStr">
+      <c r="E3" s="3" t="inlineStr">
         <is>
           <t>4 CPU
 (platform-managed)</t>
         </is>
       </c>
-      <c r="F3" s="4" t="inlineStr">
+      <c r="F3" s="3" t="inlineStr">
         <is>
           <t>1-2 vCPU
 (Docker container)</t>
@@ -1283,35 +2638,35 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="4" t="inlineStr">
+      <c r="A4" s="3" t="inlineStr">
         <is>
           <t>RAM (Minimum)</t>
         </is>
       </c>
-      <c r="B4" s="5" t="inlineStr">
+      <c r="B4" s="4" t="inlineStr">
         <is>
           <t>2 GB
 (hard floor; crashes below)</t>
         </is>
       </c>
-      <c r="C4" s="4" t="inlineStr">
+      <c r="C4" s="3" t="inlineStr">
         <is>
           <t>Not publicly specified
 (metal instances imply 32+ GB)</t>
         </is>
       </c>
-      <c r="D4" s="4" t="inlineStr">
+      <c r="D4" s="3" t="inlineStr">
         <is>
           <t>N/A (cloud-hosted)</t>
         </is>
       </c>
-      <c r="E4" s="4" t="inlineStr">
+      <c r="E4" s="3" t="inlineStr">
         <is>
           <t>8 GB + 6 GB swap
 (platform-managed)</t>
         </is>
       </c>
-      <c r="F4" s="4" t="inlineStr">
+      <c r="F4" s="3" t="inlineStr">
         <is>
           <t>2-4 GB
 (depends on tooling)</t>
@@ -1319,81 +2674,81 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="4" t="inlineStr">
+      <c r="A5" s="3" t="inlineStr">
         <is>
           <t>Storage (Minimum)</t>
         </is>
       </c>
-      <c r="B5" s="5" t="inlineStr">
+      <c r="B5" s="4" t="inlineStr">
         <is>
           <t>20 GB</t>
         </is>
       </c>
-      <c r="C5" s="4" t="inlineStr">
+      <c r="C5" s="3" t="inlineStr">
         <is>
           <t>Persistent Docker volumes
 (S3 backing)</t>
         </is>
       </c>
-      <c r="D5" s="4" t="inlineStr">
+      <c r="D5" s="3" t="inlineStr">
         <is>
           <t>N/A (cloud-hosted)</t>
         </is>
       </c>
-      <c r="E5" s="4" t="inlineStr">
+      <c r="E5" s="3" t="inlineStr">
         <is>
           <t>Not specified</t>
         </is>
       </c>
-      <c r="F5" s="4" t="inlineStr">
+      <c r="F5" s="3" t="inlineStr">
         <is>
           <t>10-20 GB</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="6" t="inlineStr">
+      <c r="A6" s="2" t="inlineStr">
         <is>
           <t>— RECOMMENDED / PRODUCTION —</t>
         </is>
       </c>
-      <c r="B6" s="6" t="inlineStr"/>
-      <c r="C6" s="6" t="inlineStr"/>
-      <c r="D6" s="6" t="inlineStr"/>
-      <c r="E6" s="6" t="inlineStr"/>
-      <c r="F6" s="6" t="inlineStr"/>
+      <c r="B6" s="2" t="inlineStr"/>
+      <c r="C6" s="2" t="inlineStr"/>
+      <c r="D6" s="2" t="inlineStr"/>
+      <c r="E6" s="2" t="inlineStr"/>
+      <c r="F6" s="2" t="inlineStr"/>
     </row>
     <row r="7">
-      <c r="A7" s="4" t="inlineStr">
+      <c r="A7" s="3" t="inlineStr">
         <is>
           <t>CPU (Recommended)</t>
         </is>
       </c>
-      <c r="B7" s="5" t="inlineStr">
+      <c r="B7" s="4" t="inlineStr">
         <is>
           <t>2-4+ vCPU</t>
         </is>
       </c>
-      <c r="C7" s="4" t="inlineStr">
+      <c r="C7" s="3" t="inlineStr">
         <is>
           <t>Auto-scaling EC2
 (enterprise-grade)</t>
         </is>
       </c>
-      <c r="D7" s="4" t="inlineStr">
+      <c r="D7" s="3" t="inlineStr">
         <is>
           <t>Thousands of GPUs
 (Composer training)
 Large Linux VMs (agent execution)</t>
         </is>
       </c>
-      <c r="E7" s="4" t="inlineStr">
+      <c r="E7" s="3" t="inlineStr">
         <is>
           <t>BYOM: any machine
 with network access</t>
         </is>
       </c>
-      <c r="F7" s="4" t="inlineStr">
+      <c r="F7" s="3" t="inlineStr">
         <is>
           <t>2-4 vCPU per agent
 (100+ parallel agents supported)</t>
@@ -1401,118 +2756,118 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="4" t="inlineStr">
+      <c r="A8" s="3" t="inlineStr">
         <is>
           <t>RAM (Recommended)</t>
         </is>
       </c>
-      <c r="B8" s="5" t="inlineStr">
+      <c r="B8" s="4" t="inlineStr">
         <is>
           <t>4-8 GB (standard)
 8-16 GB (browser automation)
 16+ GB (multi-agent / local LLM)</t>
         </is>
       </c>
-      <c r="C8" s="4" t="inlineStr">
+      <c r="C8" s="3" t="inlineStr">
         <is>
           <t>Not specified
 (sandboxed Devbox per session)</t>
         </is>
       </c>
-      <c r="D8" s="4" t="inlineStr">
+      <c r="D8" s="3" t="inlineStr">
         <is>
           <t>Not specified publicly</t>
         </is>
       </c>
-      <c r="E8" s="4" t="inlineStr">
+      <c r="E8" s="3" t="inlineStr">
         <is>
           <t>BYOM: user-defined</t>
         </is>
       </c>
-      <c r="F8" s="4" t="inlineStr">
+      <c r="F8" s="3" t="inlineStr">
         <is>
           <t>4-8 GB per agent</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="4" t="inlineStr">
+      <c r="A9" s="3" t="inlineStr">
         <is>
           <t>Storage (Recommended)</t>
         </is>
       </c>
-      <c r="B9" s="5" t="inlineStr">
+      <c r="B9" s="4" t="inlineStr">
         <is>
           <t>40-80+ GB</t>
         </is>
       </c>
-      <c r="C9" s="4" t="inlineStr">
+      <c r="C9" s="3" t="inlineStr">
         <is>
           <t>Persistent storage option
 (Large Performant tier)</t>
         </is>
       </c>
-      <c r="D9" s="4" t="inlineStr">
+      <c r="D9" s="3" t="inlineStr">
         <is>
           <t>Not specified publicly</t>
         </is>
       </c>
-      <c r="E9" s="4" t="inlineStr">
+      <c r="E9" s="3" t="inlineStr">
         <is>
           <t>BYOM: user-defined</t>
         </is>
       </c>
-      <c r="F9" s="4" t="inlineStr">
+      <c r="F9" s="3" t="inlineStr">
         <is>
           <t>20-50 GB</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="6" t="inlineStr">
+      <c r="A10" s="2" t="inlineStr">
         <is>
           <t>— GPU REQUIREMENTS —</t>
         </is>
       </c>
-      <c r="B10" s="6" t="inlineStr"/>
-      <c r="C10" s="6" t="inlineStr"/>
-      <c r="D10" s="6" t="inlineStr"/>
-      <c r="E10" s="6" t="inlineStr"/>
-      <c r="F10" s="6" t="inlineStr"/>
+      <c r="B10" s="2" t="inlineStr"/>
+      <c r="C10" s="2" t="inlineStr"/>
+      <c r="D10" s="2" t="inlineStr"/>
+      <c r="E10" s="2" t="inlineStr"/>
+      <c r="F10" s="2" t="inlineStr"/>
     </row>
     <row r="11">
-      <c r="A11" s="4" t="inlineStr">
+      <c r="A11" s="3" t="inlineStr">
         <is>
           <t>GPU Required?</t>
         </is>
       </c>
-      <c r="B11" s="5" t="inlineStr">
+      <c r="B11" s="4" t="inlineStr">
         <is>
           <t>NO for cloud LLM usage.
 YES only for local LLM inference.</t>
         </is>
       </c>
-      <c r="C11" s="4" t="inlineStr">
+      <c r="C11" s="3" t="inlineStr">
         <is>
           <t>Not disclosed.
 Likely GPU-accelerated
 on Cognition's infrastructure.</t>
         </is>
       </c>
-      <c r="D11" s="4" t="inlineStr">
+      <c r="D11" s="3" t="inlineStr">
         <is>
           <t>YES – thousands of NVIDIA GPUs
 for Composer model training.
 Not needed for end-user IDE.</t>
         </is>
       </c>
-      <c r="E11" s="4" t="inlineStr">
+      <c r="E11" s="3" t="inlineStr">
         <is>
           <t>Not required for users.
 Cloud-hosted inference.</t>
         </is>
       </c>
-      <c r="F11" s="4" t="inlineStr">
+      <c r="F11" s="3" t="inlineStr">
         <is>
           <t>NO for cloud LLM.
 Optional for local model.</t>
@@ -1520,12 +2875,12 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="4" t="inlineStr">
+      <c r="A12" s="3" t="inlineStr">
         <is>
           <t>GPU Specs (if local LLM)</t>
         </is>
       </c>
-      <c r="B12" s="5" t="inlineStr">
+      <c r="B12" s="4" t="inlineStr">
         <is>
           <t>RTX 3060 (12GB) → 8B models
 RTX 3090 (24GB) → 34B models
@@ -1535,12 +2890,12 @@
 Rule: params × 1GB VRAM (Q4)</t>
         </is>
       </c>
-      <c r="C12" s="4" t="inlineStr">
+      <c r="C12" s="3" t="inlineStr">
         <is>
           <t>N/A (proprietary infra)</t>
         </is>
       </c>
-      <c r="D12" s="4" t="inlineStr">
+      <c r="D12" s="3" t="inlineStr">
         <is>
           <t>MXFP8 MoE kernels
 with expert parallelism.
@@ -1548,12 +2903,12 @@
 Thousands of NVIDIA GPUs.</t>
         </is>
       </c>
-      <c r="E12" s="4" t="inlineStr">
+      <c r="E12" s="3" t="inlineStr">
         <is>
           <t>N/A (cloud inference)</t>
         </is>
       </c>
-      <c r="F12" s="4" t="inlineStr">
+      <c r="F12" s="3" t="inlineStr">
         <is>
           <t>Optional: depends on
 chosen local model.</t>
@@ -1561,56 +2916,56 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="6" t="inlineStr">
+      <c r="A13" s="2" t="inlineStr">
         <is>
           <t>— RUNTIME RESOURCE CONSUMPTION —</t>
         </is>
       </c>
-      <c r="B13" s="6" t="inlineStr"/>
-      <c r="C13" s="6" t="inlineStr"/>
-      <c r="D13" s="6" t="inlineStr"/>
-      <c r="E13" s="6" t="inlineStr"/>
-      <c r="F13" s="6" t="inlineStr"/>
+      <c r="B13" s="2" t="inlineStr"/>
+      <c r="C13" s="2" t="inlineStr"/>
+      <c r="D13" s="2" t="inlineStr"/>
+      <c r="E13" s="2" t="inlineStr"/>
+      <c r="F13" s="2" t="inlineStr"/>
     </row>
     <row r="14">
-      <c r="A14" s="4" t="inlineStr">
+      <c r="A14" s="3" t="inlineStr">
         <is>
           <t>Idle CPU Load</t>
         </is>
       </c>
-      <c r="B14" s="5" t="inlineStr">
+      <c r="B14" s="4" t="inlineStr">
         <is>
           <t>1-3% (background router)</t>
         </is>
       </c>
-      <c r="C14" s="4" t="inlineStr">
+      <c r="C14" s="3" t="inlineStr">
         <is>
           <t>Minimal (session-based)</t>
         </is>
       </c>
-      <c r="D14" s="4" t="inlineStr">
+      <c r="D14" s="3" t="inlineStr">
         <is>
           <t>Low (desktop IDE idle)</t>
         </is>
       </c>
-      <c r="E14" s="4" t="inlineStr">
+      <c r="E14" s="3" t="inlineStr">
         <is>
           <t>Auto-pauses when idle</t>
         </is>
       </c>
-      <c r="F14" s="4" t="inlineStr">
+      <c r="F14" s="3" t="inlineStr">
         <is>
           <t>Minimal (Docker idle)</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="4" t="inlineStr">
+      <c r="A15" s="3" t="inlineStr">
         <is>
           <t>Active CPU Load</t>
         </is>
       </c>
-      <c r="B15" s="5" t="inlineStr">
+      <c r="B15" s="4" t="inlineStr">
         <is>
           <t>Single agent + cloud LLM: minimal
 Browser automation (3 nodes): 75-90%
@@ -1618,35 +2973,35 @@
 Local 14B model: 45-60%</t>
         </is>
       </c>
-      <c r="C15" s="4" t="inlineStr">
+      <c r="C15" s="3" t="inlineStr">
         <is>
           <t>Not disclosed</t>
         </is>
       </c>
-      <c r="D15" s="4" t="inlineStr">
+      <c r="D15" s="3" t="inlineStr">
         <is>
           <t>Not disclosed
 (250 tokens/sec inference)</t>
         </is>
       </c>
-      <c r="E15" s="4" t="inlineStr">
+      <c r="E15" s="3" t="inlineStr">
         <is>
           <t>Not disclosed</t>
         </is>
       </c>
-      <c r="F15" s="4" t="inlineStr">
+      <c r="F15" s="3" t="inlineStr">
         <is>
           <t>Not disclosed</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="4" t="inlineStr">
+      <c r="A16" s="3" t="inlineStr">
         <is>
           <t>Memory Footprint</t>
         </is>
       </c>
-      <c r="B16" s="5" t="inlineStr">
+      <c r="B16" s="4" t="inlineStr">
         <is>
           <t>Node.js Gateway: 300-500 MB idle.
 Browser automation: 8 GB hard req.
@@ -1654,34 +3009,34 @@
 Local 14B model: 5.4 GB peak.</t>
         </is>
       </c>
-      <c r="C16" s="4" t="inlineStr">
+      <c r="C16" s="3" t="inlineStr">
         <is>
           <t>Not disclosed</t>
         </is>
       </c>
-      <c r="D16" s="4" t="inlineStr">
+      <c r="D16" s="3" t="inlineStr">
         <is>
           <t>Not disclosed</t>
         </is>
       </c>
-      <c r="E16" s="4" t="inlineStr">
+      <c r="E16" s="3" t="inlineStr">
         <is>
           <t>Not disclosed</t>
         </is>
       </c>
-      <c r="F16" s="4" t="inlineStr">
+      <c r="F16" s="3" t="inlineStr">
         <is>
           <t>Not disclosed</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="4" t="inlineStr">
+      <c r="A17" s="3" t="inlineStr">
         <is>
           <t>Scaling Approach</t>
         </is>
       </c>
-      <c r="B17" s="5" t="inlineStr">
+      <c r="B17" s="4" t="inlineStr">
         <is>
           <t>Single-instance by default.
 Kubernetes (ClawPod) for 1-100+ agents
@@ -1689,28 +3044,28 @@
 network policies, persistent volumes.</t>
         </is>
       </c>
-      <c r="C17" s="4" t="inlineStr">
+      <c r="C17" s="3" t="inlineStr">
         <is>
           <t>Auto-scaling EC2 instances.
 Sandboxed Devbox per session.
 Enterprise SaaS or dedicated VPC.</t>
         </is>
       </c>
-      <c r="D17" s="4" t="inlineStr">
+      <c r="D17" s="3" t="inlineStr">
         <is>
           <t>Single large Linux VM
 with shared state files.
 Thousands of agents per VM.</t>
         </is>
       </c>
-      <c r="E17" s="4" t="inlineStr">
+      <c r="E17" s="3" t="inlineStr">
         <is>
           <t>Platform-managed compute.
 Auto-pause on idle.
 BYOM for custom infra.</t>
         </is>
       </c>
-      <c r="F17" s="4" t="inlineStr">
+      <c r="F17" s="3" t="inlineStr">
         <is>
           <t>SWE-ReX framework.
 Docker containers per agent.
@@ -1724,7 +3079,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1804,47 +3159,47 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="6" t="inlineStr">
+      <c r="A2" s="2" t="inlineStr">
         <is>
           <t>— SUBSCRIPTION / LICENSE —</t>
         </is>
       </c>
-      <c r="B2" s="6" t="inlineStr"/>
-      <c r="C2" s="6" t="inlineStr"/>
-      <c r="D2" s="6" t="inlineStr"/>
-      <c r="E2" s="6" t="inlineStr"/>
-      <c r="F2" s="6" t="inlineStr"/>
-      <c r="G2" s="6" t="inlineStr"/>
-      <c r="H2" s="6" t="inlineStr"/>
-      <c r="I2" s="6" t="inlineStr"/>
-      <c r="J2" s="6" t="inlineStr"/>
-      <c r="K2" s="6" t="inlineStr"/>
+      <c r="B2" s="2" t="inlineStr"/>
+      <c r="C2" s="2" t="inlineStr"/>
+      <c r="D2" s="2" t="inlineStr"/>
+      <c r="E2" s="2" t="inlineStr"/>
+      <c r="F2" s="2" t="inlineStr"/>
+      <c r="G2" s="2" t="inlineStr"/>
+      <c r="H2" s="2" t="inlineStr"/>
+      <c r="I2" s="2" t="inlineStr"/>
+      <c r="J2" s="2" t="inlineStr"/>
+      <c r="K2" s="2" t="inlineStr"/>
     </row>
     <row r="3">
-      <c r="A3" s="4" t="inlineStr">
+      <c r="A3" s="3" t="inlineStr">
         <is>
           <t>Software License Cost</t>
         </is>
       </c>
-      <c r="B3" s="5" t="inlineStr">
+      <c r="B3" s="4" t="inlineStr">
         <is>
           <t>FREE (MIT open source)</t>
         </is>
       </c>
-      <c r="C3" s="4" t="inlineStr">
+      <c r="C3" s="3" t="inlineStr">
         <is>
           <t>$500/month (unlimited seats)
 Enterprise: custom</t>
         </is>
       </c>
-      <c r="D3" s="4" t="inlineStr">
+      <c r="D3" s="3" t="inlineStr">
         <is>
           <t>Free / $20 / $60 / $200 per month
 Teams: $40/user/mo
 Enterprise: custom</t>
         </is>
       </c>
-      <c r="E3" s="4" t="inlineStr">
+      <c r="E3" s="3" t="inlineStr">
         <is>
           <t>Pro: $10/mo
 Pro+: $39/mo
@@ -1852,7 +3207,7 @@
 Enterprise: $39/user/mo</t>
         </is>
       </c>
-      <c r="F3" s="4" t="inlineStr">
+      <c r="F3" s="3" t="inlineStr">
         <is>
           <t>Pro: $20/mo
 Max 5x: $100/mo
@@ -1860,63 +3215,63 @@
 Teams: $150/user/mo</t>
         </is>
       </c>
-      <c r="G3" s="4" t="inlineStr">
+      <c r="G3" s="3" t="inlineStr">
         <is>
           <t>Free / $15/mo
 Teams: $30/user/mo
 Enterprise: custom</t>
         </is>
       </c>
-      <c r="H3" s="4" t="inlineStr">
+      <c r="H3" s="3" t="inlineStr">
         <is>
           <t>Pro: $20/mo
 Max: $200/mo
 Enterprise: custom</t>
         </is>
       </c>
-      <c r="I3" s="4" t="inlineStr">
+      <c r="I3" s="3" t="inlineStr">
         <is>
           <t>Effort-based pricing.
 Credits per plan tier.
 Turbo mode: 6× Power cost.</t>
         </is>
       </c>
-      <c r="J3" s="4" t="inlineStr">
+      <c r="J3" s="3" t="inlineStr">
         <is>
           <t>Free: $0
 Pro: $19/user/mo</t>
         </is>
       </c>
-      <c r="K3" s="4" t="inlineStr">
+      <c r="K3" s="3" t="inlineStr">
         <is>
           <t>FREE (MIT open source)</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="6" t="inlineStr">
+      <c r="A4" s="2" t="inlineStr">
         <is>
           <t>— INFRASTRUCTURE / COMPUTE COSTS —</t>
         </is>
       </c>
-      <c r="B4" s="6" t="inlineStr"/>
-      <c r="C4" s="6" t="inlineStr"/>
-      <c r="D4" s="6" t="inlineStr"/>
-      <c r="E4" s="6" t="inlineStr"/>
-      <c r="F4" s="6" t="inlineStr"/>
-      <c r="G4" s="6" t="inlineStr"/>
-      <c r="H4" s="6" t="inlineStr"/>
-      <c r="I4" s="6" t="inlineStr"/>
-      <c r="J4" s="6" t="inlineStr"/>
-      <c r="K4" s="6" t="inlineStr"/>
+      <c r="B4" s="2" t="inlineStr"/>
+      <c r="C4" s="2" t="inlineStr"/>
+      <c r="D4" s="2" t="inlineStr"/>
+      <c r="E4" s="2" t="inlineStr"/>
+      <c r="F4" s="2" t="inlineStr"/>
+      <c r="G4" s="2" t="inlineStr"/>
+      <c r="H4" s="2" t="inlineStr"/>
+      <c r="I4" s="2" t="inlineStr"/>
+      <c r="J4" s="2" t="inlineStr"/>
+      <c r="K4" s="2" t="inlineStr"/>
     </row>
     <row r="5">
-      <c r="A5" s="4" t="inlineStr">
+      <c r="A5" s="3" t="inlineStr">
         <is>
           <t>Hosting / Compute Cost</t>
         </is>
       </c>
-      <c r="B5" s="5" t="inlineStr">
+      <c r="B5" s="4" t="inlineStr">
         <is>
           <t>Self-hosted VPS:
 Budget: $4-6/mo
@@ -1925,52 +3280,52 @@
 Free: Oracle Cloud Always Free</t>
         </is>
       </c>
-      <c r="C5" s="4" t="inlineStr">
+      <c r="C5" s="3" t="inlineStr">
         <is>
           <t>Included in subscription.
 Enterprise VPC: customer
 pays AWS infrastructure.</t>
         </is>
       </c>
-      <c r="D5" s="4" t="inlineStr">
+      <c r="D5" s="3" t="inlineStr">
         <is>
           <t>Included in subscription.
 Cloud agents included.</t>
         </is>
       </c>
-      <c r="E5" s="4" t="inlineStr">
+      <c r="E5" s="3" t="inlineStr">
         <is>
           <t>Included in subscription.</t>
         </is>
       </c>
-      <c r="F5" s="4" t="inlineStr">
+      <c r="F5" s="3" t="inlineStr">
         <is>
           <t>Included in subscription
 (or API pay-as-you-go).</t>
         </is>
       </c>
-      <c r="G5" s="4" t="inlineStr">
+      <c r="G5" s="3" t="inlineStr">
         <is>
           <t>Included in subscription.</t>
         </is>
       </c>
-      <c r="H5" s="4" t="inlineStr">
+      <c r="H5" s="3" t="inlineStr">
         <is>
           <t>Included (platform-managed)
 or BYOM (user-paid infra).</t>
         </is>
       </c>
-      <c r="I5" s="4" t="inlineStr">
+      <c r="I5" s="3" t="inlineStr">
         <is>
           <t>Included in subscription.</t>
         </is>
       </c>
-      <c r="J5" s="4" t="inlineStr">
+      <c r="J5" s="3" t="inlineStr">
         <is>
           <t>Included in subscription.</t>
         </is>
       </c>
-      <c r="K5" s="4" t="inlineStr">
+      <c r="K5" s="3" t="inlineStr">
         <is>
           <t>Self-hosted: $4-24/mo
 (VPS) or free (local Docker).</t>
@@ -1978,13 +3333,13 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="4" t="inlineStr">
+      <c r="A6" s="3" t="inlineStr">
         <is>
           <t>LLM / API Costs
 (variable)</t>
         </is>
       </c>
-      <c r="B6" s="5" t="inlineStr">
+      <c r="B6" s="4" t="inlineStr">
         <is>
           <t>$5-200+/month
 depends on model &amp; usage.
@@ -1992,57 +3347,57 @@
 DeepSeek/Gemini Flash: $5-10/mo.</t>
         </is>
       </c>
-      <c r="C6" s="4" t="inlineStr">
+      <c r="C6" s="3" t="inlineStr">
         <is>
           <t>Included in subscription.</t>
         </is>
       </c>
-      <c r="D6" s="4" t="inlineStr">
+      <c r="D6" s="3" t="inlineStr">
         <is>
           <t>Included within credit pool.
 Overages billed per usage.</t>
         </is>
       </c>
-      <c r="E6" s="4" t="inlineStr">
+      <c r="E6" s="3" t="inlineStr">
         <is>
           <t>Included.
 Premium requests: $0.04 each
 (overage).</t>
         </is>
       </c>
-      <c r="F6" s="4" t="inlineStr">
+      <c r="F6" s="3" t="inlineStr">
         <is>
           <t>API: $3-25/M tokens
 (varies by model).
 Subscription: included.</t>
         </is>
       </c>
-      <c r="G6" s="4" t="inlineStr">
+      <c r="G6" s="3" t="inlineStr">
         <is>
           <t>Included within credits.
 Add-on: $10/250 credits.</t>
         </is>
       </c>
-      <c r="H6" s="4" t="inlineStr">
+      <c r="H6" s="3" t="inlineStr">
         <is>
           <t>Included within tokens.
 Overage: $2.70/M tokens.</t>
         </is>
       </c>
-      <c r="I6" s="4" t="inlineStr">
+      <c r="I6" s="3" t="inlineStr">
         <is>
           <t>Included within credits.
 Effort-based pricing.</t>
         </is>
       </c>
-      <c r="J6" s="4" t="inlineStr">
+      <c r="J6" s="3" t="inlineStr">
         <is>
           <t>Included.
 Code transformation:
 $0.003/line (overage).</t>
         </is>
       </c>
-      <c r="K6" s="4" t="inlineStr">
+      <c r="K6" s="3" t="inlineStr">
         <is>
           <t>User pays own API costs.
 Model-agnostic.</t>
@@ -2050,78 +3405,78 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="6" t="inlineStr">
+      <c r="A7" s="2" t="inlineStr">
         <is>
           <t>— TOTAL COST OF OWNERSHIP (TCO) —</t>
         </is>
       </c>
-      <c r="B7" s="6" t="inlineStr"/>
-      <c r="C7" s="6" t="inlineStr"/>
-      <c r="D7" s="6" t="inlineStr"/>
-      <c r="E7" s="6" t="inlineStr"/>
-      <c r="F7" s="6" t="inlineStr"/>
-      <c r="G7" s="6" t="inlineStr"/>
-      <c r="H7" s="6" t="inlineStr"/>
-      <c r="I7" s="6" t="inlineStr"/>
-      <c r="J7" s="6" t="inlineStr"/>
-      <c r="K7" s="6" t="inlineStr"/>
+      <c r="B7" s="2" t="inlineStr"/>
+      <c r="C7" s="2" t="inlineStr"/>
+      <c r="D7" s="2" t="inlineStr"/>
+      <c r="E7" s="2" t="inlineStr"/>
+      <c r="F7" s="2" t="inlineStr"/>
+      <c r="G7" s="2" t="inlineStr"/>
+      <c r="H7" s="2" t="inlineStr"/>
+      <c r="I7" s="2" t="inlineStr"/>
+      <c r="J7" s="2" t="inlineStr"/>
+      <c r="K7" s="2" t="inlineStr"/>
     </row>
     <row r="8">
-      <c r="A8" s="4" t="inlineStr">
+      <c r="A8" s="3" t="inlineStr">
         <is>
           <t>Light Usage
 (individual, occasional)</t>
         </is>
       </c>
-      <c r="B8" s="5" t="inlineStr">
+      <c r="B8" s="4" t="inlineStr">
         <is>
           <t>$10-22/month
 (VPS + cheap model APIs)</t>
         </is>
       </c>
-      <c r="C8" s="4" t="inlineStr">
+      <c r="C8" s="3" t="inlineStr">
         <is>
           <t>$500/month</t>
         </is>
       </c>
-      <c r="D8" s="4" t="inlineStr">
+      <c r="D8" s="3" t="inlineStr">
         <is>
           <t>$0-20/month</t>
         </is>
       </c>
-      <c r="E8" s="4" t="inlineStr">
+      <c r="E8" s="3" t="inlineStr">
         <is>
           <t>$10-19/month</t>
         </is>
       </c>
-      <c r="F8" s="4" t="inlineStr">
+      <c r="F8" s="3" t="inlineStr">
         <is>
           <t>$20/month (Pro)</t>
         </is>
       </c>
-      <c r="G8" s="4" t="inlineStr">
+      <c r="G8" s="3" t="inlineStr">
         <is>
           <t>$0-15/month</t>
         </is>
       </c>
-      <c r="H8" s="4" t="inlineStr">
+      <c r="H8" s="3" t="inlineStr">
         <is>
           <t>$20/month</t>
         </is>
       </c>
-      <c r="I8" s="4" t="inlineStr">
+      <c r="I8" s="3" t="inlineStr">
         <is>
           <t>~$5-25/month
 (effort-based)</t>
         </is>
       </c>
-      <c r="J8" s="4" t="inlineStr">
+      <c r="J8" s="3" t="inlineStr">
         <is>
           <t>$0 (Free tier:
 50 agentic requests)</t>
         </is>
       </c>
-      <c r="K8" s="4" t="inlineStr">
+      <c r="K8" s="3" t="inlineStr">
         <is>
           <t>$0-10/month
 (local + API costs)</t>
@@ -2129,129 +3484,129 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="4" t="inlineStr">
+      <c r="A9" s="3" t="inlineStr">
         <is>
           <t>Moderate Usage
 (daily professional use)</t>
         </is>
       </c>
-      <c r="B9" s="5" t="inlineStr">
+      <c r="B9" s="4" t="inlineStr">
         <is>
           <t>$27-72/month
 (VPS + moderate API)</t>
         </is>
       </c>
-      <c r="C9" s="4" t="inlineStr">
+      <c r="C9" s="3" t="inlineStr">
         <is>
           <t>$500/month</t>
         </is>
       </c>
-      <c r="D9" s="4" t="inlineStr">
+      <c r="D9" s="3" t="inlineStr">
         <is>
           <t>$60/month (Pro+)</t>
         </is>
       </c>
-      <c r="E9" s="4" t="inlineStr">
+      <c r="E9" s="3" t="inlineStr">
         <is>
           <t>$39/month (Pro+)</t>
         </is>
       </c>
-      <c r="F9" s="4" t="inlineStr">
+      <c r="F9" s="3" t="inlineStr">
         <is>
           <t>$100-200/month (Max)</t>
         </is>
       </c>
-      <c r="G9" s="4" t="inlineStr">
+      <c r="G9" s="3" t="inlineStr">
         <is>
           <t>$15-30/month</t>
         </is>
       </c>
-      <c r="H9" s="4" t="inlineStr">
+      <c r="H9" s="3" t="inlineStr">
         <is>
           <t>$200/month (Max)</t>
         </is>
       </c>
-      <c r="I9" s="4" t="inlineStr">
+      <c r="I9" s="3" t="inlineStr">
         <is>
           <t>~$50-150/month</t>
         </is>
       </c>
-      <c r="J9" s="4" t="inlineStr">
+      <c r="J9" s="3" t="inlineStr">
         <is>
           <t>$19/month (Pro)</t>
         </is>
       </c>
-      <c r="K9" s="4" t="inlineStr">
+      <c r="K9" s="3" t="inlineStr">
         <is>
           <t>$10-50/month</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="4" t="inlineStr">
+      <c r="A10" s="3" t="inlineStr">
         <is>
           <t>Heavy / Enterprise
 (multi-agent, team)</t>
         </is>
       </c>
-      <c r="B10" s="5" t="inlineStr">
+      <c r="B10" s="4" t="inlineStr">
         <is>
           <t>$62-224+/month per instance.
 Per-person: $300-500/mo/agent.
 100 people: $30-50K/mo.</t>
         </is>
       </c>
-      <c r="C10" s="4" t="inlineStr">
+      <c r="C10" s="3" t="inlineStr">
         <is>
           <t>$500/mo + enterprise pricing.
 Enterprise: Goldman Sachs,
 Santander, Nubank.</t>
         </is>
       </c>
-      <c r="D10" s="4" t="inlineStr">
+      <c r="D10" s="3" t="inlineStr">
         <is>
           <t>$200/mo (Ultra) or
 $40/user/mo (Teams).
 Enterprise: custom.</t>
         </is>
       </c>
-      <c r="E10" s="4" t="inlineStr">
+      <c r="E10" s="3" t="inlineStr">
         <is>
           <t>$39/user/mo (Enterprise).
 Volume discounts available.</t>
         </is>
       </c>
-      <c r="F10" s="4" t="inlineStr">
+      <c r="F10" s="3" t="inlineStr">
         <is>
           <t>$150/user/mo (Teams).
 Enterprise: custom.</t>
         </is>
       </c>
-      <c r="G10" s="4" t="inlineStr">
+      <c r="G10" s="3" t="inlineStr">
         <is>
           <t>$30/user/mo (Teams).
 Enterprise: custom.</t>
         </is>
       </c>
-      <c r="H10" s="4" t="inlineStr">
+      <c r="H10" s="3" t="inlineStr">
         <is>
           <t>Enterprise: custom pricing.
 Unlimited features.</t>
         </is>
       </c>
-      <c r="I10" s="4" t="inlineStr">
+      <c r="I10" s="3" t="inlineStr">
         <is>
           <t>Pro plan + high usage.
 Enterprise: custom.</t>
         </is>
       </c>
-      <c r="J10" s="4" t="inlineStr">
+      <c r="J10" s="3" t="inlineStr">
         <is>
           <t>$19/user/mo.
 Volume discounts.</t>
         </is>
       </c>
-      <c r="K10" s="4" t="inlineStr">
+      <c r="K10" s="3" t="inlineStr">
         <is>
           <t>$20-100+/month
 (infra + API costs).</t>
@@ -2259,29 +3614,29 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="6" t="inlineStr">
+      <c r="A11" s="2" t="inlineStr">
         <is>
           <t>— HIDDEN / ADDITIONAL COSTS —</t>
         </is>
       </c>
-      <c r="B11" s="6" t="inlineStr"/>
-      <c r="C11" s="6" t="inlineStr"/>
-      <c r="D11" s="6" t="inlineStr"/>
-      <c r="E11" s="6" t="inlineStr"/>
-      <c r="F11" s="6" t="inlineStr"/>
-      <c r="G11" s="6" t="inlineStr"/>
-      <c r="H11" s="6" t="inlineStr"/>
-      <c r="I11" s="6" t="inlineStr"/>
-      <c r="J11" s="6" t="inlineStr"/>
-      <c r="K11" s="6" t="inlineStr"/>
+      <c r="B11" s="2" t="inlineStr"/>
+      <c r="C11" s="2" t="inlineStr"/>
+      <c r="D11" s="2" t="inlineStr"/>
+      <c r="E11" s="2" t="inlineStr"/>
+      <c r="F11" s="2" t="inlineStr"/>
+      <c r="G11" s="2" t="inlineStr"/>
+      <c r="H11" s="2" t="inlineStr"/>
+      <c r="I11" s="2" t="inlineStr"/>
+      <c r="J11" s="2" t="inlineStr"/>
+      <c r="K11" s="2" t="inlineStr"/>
     </row>
     <row r="12">
-      <c r="A12" s="4" t="inlineStr">
+      <c r="A12" s="3" t="inlineStr">
         <is>
           <t>Hidden Costs</t>
         </is>
       </c>
-      <c r="B12" s="5" t="inlineStr">
+      <c r="B12" s="4" t="inlineStr">
         <is>
           <t>System prompt token burn: $5-30/mo.
 Heartbeat checks: $0-90/mo.
@@ -2289,60 +3644,60 @@
 Model switching overhead.</t>
         </is>
       </c>
-      <c r="C12" s="4" t="inlineStr">
+      <c r="C12" s="3" t="inlineStr">
         <is>
           <t>AWS VPC infra costs (enterprise).
 Data transfer charges.
 Onboarding/integration time.</t>
         </is>
       </c>
-      <c r="D12" s="4" t="inlineStr">
+      <c r="D12" s="3" t="inlineStr">
         <is>
           <t>Overage charges beyond
 credit pool.
 Bugbot add-on: $40/user/mo.</t>
         </is>
       </c>
-      <c r="E12" s="4" t="inlineStr">
+      <c r="E12" s="3" t="inlineStr">
         <is>
           <t>Premium request overages
 ($0.04/request).
 Model upgrade costs.</t>
         </is>
       </c>
-      <c r="F12" s="4" t="inlineStr">
+      <c r="F12" s="3" t="inlineStr">
         <is>
           <t>Token-based billing can
 spike unexpectedly.
 No caching = 4x cost.</t>
         </is>
       </c>
-      <c r="G12" s="4" t="inlineStr">
+      <c r="G12" s="3" t="inlineStr">
         <is>
           <t>Credit overage ($10/250).
 Model-specific multipliers.</t>
         </is>
       </c>
-      <c r="H12" s="4" t="inlineStr">
+      <c r="H12" s="3" t="inlineStr">
         <is>
           <t>Token overage: $2.70/M.
 Cached vs. uncached pricing.</t>
         </is>
       </c>
-      <c r="I12" s="4" t="inlineStr">
+      <c r="I12" s="3" t="inlineStr">
         <is>
           <t>Turbo mode: up to 6×
 Power mode cost.
 Complex task surcharges.</t>
         </is>
       </c>
-      <c r="J12" s="4" t="inlineStr">
+      <c r="J12" s="3" t="inlineStr">
         <is>
           <t>Code transformation
 overage: $0.003/line.</t>
         </is>
       </c>
-      <c r="K12" s="4" t="inlineStr">
+      <c r="K12" s="3" t="inlineStr">
         <is>
           <t>API costs are unbounded.
 Infra maintenance time.</t>
@@ -2354,7 +3709,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2410,12 +3765,12 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="5" t="inlineStr">
+      <c r="A2" s="4" t="inlineStr">
         <is>
           <t>OpenClaw</t>
         </is>
       </c>
-      <c r="B2" s="5" t="inlineStr">
+      <c r="B2" s="4" t="inlineStr">
         <is>
           <t>Open-source, self-hosted, model-agnostic
 personal AI assistant.
@@ -2424,14 +3779,14 @@
 Lowest TCO at scale.</t>
         </is>
       </c>
-      <c r="C2" s="5" t="inlineStr">
+      <c r="C2" s="4" t="inlineStr">
         <is>
           <t>Power users, privacy-conscious,
 SMBs wanting automation
 without vendor lock-in.</t>
         </is>
       </c>
-      <c r="D2" s="5" t="inlineStr">
+      <c r="D2" s="4" t="inlineStr">
         <is>
           <t>322K+ GitHub stars.
 Fastest-growing GH project ever.
@@ -2439,7 +3794,7 @@
 Model-agnostic flexibility.</t>
         </is>
       </c>
-      <c r="E2" s="5" t="inlineStr">
+      <c r="E2" s="4" t="inlineStr">
         <is>
           <t>NOT a coding agent (general assistant).
 Self-hosting maintenance burden.
@@ -2447,13 +3802,13 @@
 API costs can spike with expensive models.</t>
         </is>
       </c>
-      <c r="F2" s="5" t="inlineStr">
+      <c r="F2" s="4" t="inlineStr">
         <is>
           <t>FULL – data never leaves
 user's infrastructure.</t>
         </is>
       </c>
-      <c r="G2" s="5" t="inlineStr">
+      <c r="G2" s="4" t="inlineStr">
         <is>
           <t>322K stars, 62K forks,
 360 contributors.
@@ -2463,12 +3818,12 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="4" t="inlineStr">
+      <c r="A3" s="3" t="inlineStr">
         <is>
           <t>Devin (Cognition)</t>
         </is>
       </c>
-      <c r="B3" s="4" t="inlineStr">
+      <c r="B3" s="3" t="inlineStr">
         <is>
           <t>Fully autonomous SW engineer.
 Compound AI architecture
@@ -2476,7 +3831,7 @@
 10M+ token context (Enterprise).</t>
         </is>
       </c>
-      <c r="C3" s="4" t="inlineStr">
+      <c r="C3" s="3" t="inlineStr">
         <is>
           <t>Engineering teams wanting
 asynchronous task execution.
@@ -2484,7 +3839,7 @@
 (Goldman Sachs, Santander).</t>
         </is>
       </c>
-      <c r="D3" s="4" t="inlineStr">
+      <c r="D3" s="3" t="inlineStr">
         <is>
           <t>Proprietary compound AI system.
 Enterprise relationships.
@@ -2492,7 +3847,7 @@
 Acquired Windsurf/Codeium.</t>
         </is>
       </c>
-      <c r="E3" s="4" t="inlineStr">
+      <c r="E3" s="3" t="inlineStr">
         <is>
           <t>High cost ($500/mo baseline).
 No open-source alternative.
@@ -2500,14 +3855,14 @@
 Vendor lock-in.</t>
         </is>
       </c>
-      <c r="F3" s="4" t="inlineStr">
+      <c r="F3" s="3" t="inlineStr">
         <is>
           <t>SaaS (multi-tenant) or
 customer-dedicated VPC.
 AWS PrivateLink option.</t>
         </is>
       </c>
-      <c r="G3" s="4" t="inlineStr">
+      <c r="G3" s="3" t="inlineStr">
         <is>
           <t>Major enterprise customers.
 Acquired Windsurf.
@@ -2516,12 +3871,12 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="4" t="inlineStr">
+      <c r="A4" s="3" t="inlineStr">
         <is>
           <t>Cursor</t>
         </is>
       </c>
-      <c r="B4" s="4" t="inlineStr">
+      <c r="B4" s="3" t="inlineStr">
         <is>
           <t>AI-native IDE with custom
 Composer MoE model.
@@ -2529,7 +3884,7 @@
 Sub-agent spawning.</t>
         </is>
       </c>
-      <c r="C4" s="4" t="inlineStr">
+      <c r="C4" s="3" t="inlineStr">
         <is>
           <t>Senior developers wanting
 flow-state amplification.
@@ -2537,7 +3892,7 @@
 AI-powered workflows.</t>
         </is>
       </c>
-      <c r="D4" s="4" t="inlineStr">
+      <c r="D4" s="3" t="inlineStr">
         <is>
           <t>Custom-trained Composer model.
 250 tokens/sec inference.
@@ -2545,7 +3900,7 @@
 Largest AI IDE user base.</t>
         </is>
       </c>
-      <c r="E4" s="4" t="inlineStr">
+      <c r="E4" s="3" t="inlineStr">
         <is>
           <t>Not fully autonomous
 (IDE-dependent).
@@ -2553,14 +3908,14 @@
 be unpredictable.</t>
         </is>
       </c>
-      <c r="F4" s="4" t="inlineStr">
+      <c r="F4" s="3" t="inlineStr">
         <is>
           <t>Local IDE + cloud inference.
 Code stays local;
 prompts sent to cloud.</t>
         </is>
       </c>
-      <c r="G4" s="4" t="inlineStr">
+      <c r="G4" s="3" t="inlineStr">
         <is>
           <t>Dominant AI IDE.
 Rapidly growing Teams/Enterprise.</t>
@@ -2568,26 +3923,26 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="4" t="inlineStr">
+      <c r="A5" s="3" t="inlineStr">
         <is>
           <t>GitHub Copilot</t>
         </is>
       </c>
-      <c r="B5" s="4" t="inlineStr">
+      <c r="B5" s="3" t="inlineStr">
         <is>
           <t>Deepest GitHub integration.
 Issue → PR workflow.
 Largest enterprise installed base.</t>
         </is>
       </c>
-      <c r="C5" s="4" t="inlineStr">
+      <c r="C5" s="3" t="inlineStr">
         <is>
           <t>Enterprise teams already
 on GitHub ecosystem.
 Compliance-focused orgs.</t>
         </is>
       </c>
-      <c r="D5" s="4" t="inlineStr">
+      <c r="D5" s="3" t="inlineStr">
         <is>
           <t>GitHub ecosystem lock-in.
 Microsoft/OpenAI backing.
@@ -2595,21 +3950,21 @@
 IP indemnity.</t>
         </is>
       </c>
-      <c r="E5" s="4" t="inlineStr">
+      <c r="E5" s="3" t="inlineStr">
         <is>
           <t>Lower autonomy than Devin.
 Premium request limits.
 Less flexible model choice.</t>
         </is>
       </c>
-      <c r="F5" s="4" t="inlineStr">
+      <c r="F5" s="3" t="inlineStr">
         <is>
           <t>Cloud SaaS.
 Microsoft enterprise
 compliance certifications.</t>
         </is>
       </c>
-      <c r="G5" s="4" t="inlineStr">
+      <c r="G5" s="3" t="inlineStr">
         <is>
           <t>Largest installed base among
 AI coding tools.
@@ -2618,12 +3973,12 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="4" t="inlineStr">
+      <c r="A6" s="3" t="inlineStr">
         <is>
           <t>Claude Code</t>
         </is>
       </c>
-      <c r="B6" s="4" t="inlineStr">
+      <c r="B6" s="3" t="inlineStr">
         <is>
           <t>Highest SWE-bench score
 (79.6-82%).
@@ -2631,14 +3986,14 @@
 84% prompt cache hit rate.</t>
         </is>
       </c>
-      <c r="C6" s="4" t="inlineStr">
+      <c r="C6" s="3" t="inlineStr">
         <is>
           <t>Expert developers wanting
 top code quality.
 Terminal-first workflows.</t>
         </is>
       </c>
-      <c r="D6" s="4" t="inlineStr">
+      <c r="D6" s="3" t="inlineStr">
         <is>
           <t>Highest benchmark scores.
 46% developer satisfaction
@@ -2646,7 +4001,7 @@
 Anthropic model quality.</t>
         </is>
       </c>
-      <c r="E6" s="4" t="inlineStr">
+      <c r="E6" s="3" t="inlineStr">
         <is>
           <t>No self-hosting.
 Claude-only (no model choice).
@@ -2654,13 +4009,13 @@
 No IDE integration.</t>
         </is>
       </c>
-      <c r="F6" s="4" t="inlineStr">
+      <c r="F6" s="3" t="inlineStr">
         <is>
           <t>Cloud only.
 Anthropic handles all data.</t>
         </is>
       </c>
-      <c r="G6" s="4" t="inlineStr">
+      <c r="G6" s="3" t="inlineStr">
         <is>
           <t>Most-loved AI coding tool
 in 2026 (46% satisfaction).</t>
@@ -2668,12 +4023,12 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="4" t="inlineStr">
+      <c r="A7" s="3" t="inlineStr">
         <is>
           <t>Windsurf</t>
         </is>
       </c>
-      <c r="B7" s="4" t="inlineStr">
+      <c r="B7" s="3" t="inlineStr">
         <is>
           <t>SWE-1.5 at 950 tokens/sec
 (13× Sonnet, 6× Haiku).
@@ -2681,35 +4036,35 @@
 Persistent Memories.</t>
         </is>
       </c>
-      <c r="C7" s="4" t="inlineStr">
+      <c r="C7" s="3" t="inlineStr">
         <is>
           <t>Developers wanting fast,
 context-aware IDE assistance.
 40+ IDE support.</t>
         </is>
       </c>
-      <c r="D7" s="4" t="inlineStr">
+      <c r="D7" s="3" t="inlineStr">
         <is>
           <t>Fastest inference speed.
 Cognition (Devin) backing.
 Broad IDE compatibility.</t>
         </is>
       </c>
-      <c r="E7" s="4" t="inlineStr">
+      <c r="E7" s="3" t="inlineStr">
         <is>
           <t>Acquired by Cognition –
 future direction uncertain.
 Proprietary model dependency.</t>
         </is>
       </c>
-      <c r="F7" s="4" t="inlineStr">
+      <c r="F7" s="3" t="inlineStr">
         <is>
           <t>Local IDE + cloud inference.
 Persistent memory vectors
 stored locally.</t>
         </is>
       </c>
-      <c r="G7" s="4" t="inlineStr">
+      <c r="G7" s="3" t="inlineStr">
         <is>
           <t>800K+ active users.
 $82M ARR by mid-2025.</t>
@@ -2717,46 +4072,46 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="4" t="inlineStr">
+      <c r="A8" s="3" t="inlineStr">
         <is>
           <t>Factory AI</t>
         </is>
       </c>
-      <c r="B8" s="4" t="inlineStr">
+      <c r="B8" s="3" t="inlineStr">
         <is>
           <t>HyperCode codebase representation.
 ByteRank retrieval.
 Custom Droids (subagents).</t>
         </is>
       </c>
-      <c r="C8" s="4" t="inlineStr">
+      <c r="C8" s="3" t="inlineStr">
         <is>
           <t>Teams wanting specialized
 autonomous agents per task.
 CI/CD integration focus.</t>
         </is>
       </c>
-      <c r="D8" s="4" t="inlineStr">
+      <c r="D8" s="3" t="inlineStr">
         <is>
           <t>Multi-model task routing.
 Custom subagent architecture.
 Token-based pricing model.</t>
         </is>
       </c>
-      <c r="E8" s="4" t="inlineStr">
+      <c r="E8" s="3" t="inlineStr">
         <is>
           <t>Smaller ecosystem.
 Token overage can be costly.
 Less brand recognition.</t>
         </is>
       </c>
-      <c r="F8" s="4" t="inlineStr">
+      <c r="F8" s="3" t="inlineStr">
         <is>
           <t>Cloud SaaS or BYOM.
 BYOM keeps data local.</t>
         </is>
       </c>
-      <c r="G8" s="4" t="inlineStr">
+      <c r="G8" s="3" t="inlineStr">
         <is>
           <t>Growing but smaller
 than major competitors.</t>
@@ -2764,12 +4119,12 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="4" t="inlineStr">
+      <c r="A9" s="3" t="inlineStr">
         <is>
           <t>Replit Agent</t>
         </is>
       </c>
-      <c r="B9" s="4" t="inlineStr">
+      <c r="B9" s="3" t="inlineStr">
         <is>
           <t>Full-stack app builder
 from natural language.
@@ -2777,34 +4132,34 @@
 Design-to-code.</t>
         </is>
       </c>
-      <c r="C9" s="4" t="inlineStr">
+      <c r="C9" s="3" t="inlineStr">
         <is>
           <t>Non-technical users,
 prototypers, indie hackers.
 Rapid MVP builders.</t>
         </is>
       </c>
-      <c r="D9" s="4" t="inlineStr">
+      <c r="D9" s="3" t="inlineStr">
         <is>
           <t>End-to-end build + deploy.
 Lowest barrier to entry.
 No local setup required.</t>
         </is>
       </c>
-      <c r="E9" s="4" t="inlineStr">
+      <c r="E9" s="3" t="inlineStr">
         <is>
           <t>Limited for complex codebases.
 Effort-based pricing unpredictable.
 Not for enterprise SW engineering.</t>
         </is>
       </c>
-      <c r="F9" s="4" t="inlineStr">
+      <c r="F9" s="3" t="inlineStr">
         <is>
           <t>Cloud SaaS.
 All code on Replit servers.</t>
         </is>
       </c>
-      <c r="G9" s="4" t="inlineStr">
+      <c r="G9" s="3" t="inlineStr">
         <is>
           <t>Popular with beginners
 and prototypers.</t>
@@ -2812,26 +4167,26 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="4" t="inlineStr">
+      <c r="A10" s="3" t="inlineStr">
         <is>
           <t>Amazon Q Developer</t>
         </is>
       </c>
-      <c r="B10" s="4" t="inlineStr">
+      <c r="B10" s="3" t="inlineStr">
         <is>
           <t>Deep AWS service integration.
 Java upgrade automation.
 IP indemnity.</t>
         </is>
       </c>
-      <c r="C10" s="4" t="inlineStr">
+      <c r="C10" s="3" t="inlineStr">
         <is>
           <t>AWS-native teams.
 Java enterprise shops.
 Compliance-focused orgs.</t>
         </is>
       </c>
-      <c r="D10" s="4" t="inlineStr">
+      <c r="D10" s="3" t="inlineStr">
         <is>
           <t>AWS ecosystem integration.
 Amazon backing.
@@ -2839,20 +4194,20 @@
 IP indemnity.</t>
         </is>
       </c>
-      <c r="E10" s="4" t="inlineStr">
+      <c r="E10" s="3" t="inlineStr">
         <is>
           <t>AWS-centric (limited outside AWS).
 Smaller agentic capability
 vs. Devin/Claude Code.</t>
         </is>
       </c>
-      <c r="F10" s="4" t="inlineStr">
+      <c r="F10" s="3" t="inlineStr">
         <is>
           <t>Cloud SaaS.
 AWS enterprise compliance.</t>
         </is>
       </c>
-      <c r="G10" s="4" t="inlineStr">
+      <c r="G10" s="3" t="inlineStr">
         <is>
           <t>Growing within AWS
 customer base.</t>
@@ -2860,12 +4215,12 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="4" t="inlineStr">
+      <c r="A11" s="3" t="inlineStr">
         <is>
           <t>SWE-agent (OSS)</t>
         </is>
       </c>
-      <c r="B11" s="4" t="inlineStr">
+      <c r="B11" s="3" t="inlineStr">
         <is>
           <t>Research-grade open-source.
 100-line mini-swe-agent.
@@ -2873,34 +4228,34 @@
 Massively parallel execution.</t>
         </is>
       </c>
-      <c r="C11" s="4" t="inlineStr">
+      <c r="C11" s="3" t="inlineStr">
         <is>
           <t>Researchers, OSS contributors.
 Teams wanting full control
 over agent behavior.</t>
         </is>
       </c>
-      <c r="D11" s="4" t="inlineStr">
+      <c r="D11" s="3" t="inlineStr">
         <is>
           <t>Fully open-source.
 Research pedigree (Princeton/Stanford).
 Simplest architecture.</t>
         </is>
       </c>
-      <c r="E11" s="4" t="inlineStr">
+      <c r="E11" s="3" t="inlineStr">
         <is>
           <t>Maintenance-only mode.
 No commercial support.
 Requires technical expertise.</t>
         </is>
       </c>
-      <c r="F11" s="4" t="inlineStr">
+      <c r="F11" s="3" t="inlineStr">
         <is>
           <t>FULL – self-hosted.
 All data stays local.</t>
         </is>
       </c>
-      <c r="G11" s="4" t="inlineStr">
+      <c r="G11" s="3" t="inlineStr">
         <is>
           <t>Influential research project.
 Shifting to mini-swe-agent.</t>
@@ -2912,7 +4267,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2938,356 +4293,356 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="6" t="inlineStr">
+      <c r="A2" s="2" t="inlineStr">
         <is>
           <t>— IDENTITY —</t>
         </is>
       </c>
-      <c r="B2" s="6" t="inlineStr"/>
+      <c r="B2" s="2" t="inlineStr"/>
     </row>
     <row r="3">
-      <c r="A3" s="4" t="inlineStr">
+      <c r="A3" s="3" t="inlineStr">
         <is>
           <t>What It Is</t>
         </is>
       </c>
-      <c r="B3" s="4" t="inlineStr">
+      <c r="B3" s="3" t="inlineStr">
         <is>
           <t>Open-source, self-hosted personal AI assistant designed to take actions (not just answer questions). Connects to messaging apps (WhatsApp, Telegram, Slack, Discord, Signal, iMessage) and executes real tasks.</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="4" t="inlineStr">
+      <c r="A4" s="3" t="inlineStr">
         <is>
           <t>GitHub Stats</t>
         </is>
       </c>
-      <c r="B4" s="4" t="inlineStr">
+      <c r="B4" s="3" t="inlineStr">
         <is>
           <t>322,031 stars | 61,928 forks | 360 contributors | TypeScript 87.8% | MIT License | 68 releases (latest v2026.3.13-1)</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="4" t="inlineStr">
+      <c r="A5" s="3" t="inlineStr">
         <is>
           <t>Growth Milestone</t>
         </is>
       </c>
-      <c r="B5" s="4" t="inlineStr">
+      <c r="B5" s="3" t="inlineStr">
         <is>
           <t>Fastest-growing project in GitHub history. Surpassed React's star count in ~60 days (React took 13 years). 300,000-400,000 users worldwide by March 2026.</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="6" t="inlineStr">
+      <c r="A6" s="2" t="inlineStr">
         <is>
           <t>— ARCHITECTURE —</t>
         </is>
       </c>
-      <c r="B6" s="6" t="inlineStr"/>
+      <c r="B6" s="2" t="inlineStr"/>
     </row>
     <row r="7">
-      <c r="A7" s="4" t="inlineStr">
+      <c r="A7" s="3" t="inlineStr">
         <is>
           <t>Runtime</t>
         </is>
       </c>
-      <c r="B7" s="4" t="inlineStr">
+      <c r="B7" s="3" t="inlineStr">
         <is>
           <t>Node.js long-running daemon process (Gateway). Handles message routing, session persistence, cron jobs, and tool execution.</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="4" t="inlineStr">
+      <c r="A8" s="3" t="inlineStr">
         <is>
           <t>I/O Profile</t>
         </is>
       </c>
-      <c r="B8" s="4" t="inlineStr">
+      <c r="B8" s="3" t="inlineStr">
         <is>
           <t>I/O bound when using cloud LLM APIs. Becomes CPU-intensive during tool execution, browser automation, and local LLM inference.</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="4" t="inlineStr">
+      <c r="A9" s="3" t="inlineStr">
         <is>
           <t>MCP Integration</t>
         </is>
       </c>
-      <c r="B9" s="4" t="inlineStr">
+      <c r="B9" s="3" t="inlineStr">
         <is>
           <t>3,200+ MCP skills on ClawHub marketplace. Hot-reloading plugins. Cryptographic message signing (ECDSA P-256) for MCP transport security.</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="4" t="inlineStr">
+      <c r="A10" s="3" t="inlineStr">
         <is>
           <t>Multi-Agent Patterns</t>
         </is>
       </c>
-      <c r="B10" s="4" t="inlineStr">
+      <c r="B10" s="3" t="inlineStr">
         <is>
           <t>Per-Function (most cost-effective), Agent Teams (coordinated specialists), Hierarchical (chief-of-staff orchestrator). Single-instance by default; Kubernetes (ClawPod) for 1-100+ agents.</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="6" t="inlineStr">
+      <c r="A11" s="2" t="inlineStr">
         <is>
           <t>— MINIMUM COMPUTE —</t>
         </is>
       </c>
-      <c r="B11" s="6" t="inlineStr"/>
+      <c r="B11" s="2" t="inlineStr"/>
     </row>
     <row r="12">
-      <c r="A12" s="4" t="inlineStr">
+      <c r="A12" s="3" t="inlineStr">
         <is>
           <t>Testing / Light</t>
         </is>
       </c>
-      <c r="B12" s="4" t="inlineStr">
+      <c r="B12" s="3" t="inlineStr">
         <is>
           <t>1-2 vCPU | 2 GB RAM | 20 GB storage</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="4" t="inlineStr">
+      <c r="A13" s="3" t="inlineStr">
         <is>
           <t>Daily Use (Recommended)</t>
         </is>
       </c>
-      <c r="B13" s="4" t="inlineStr">
+      <c r="B13" s="3" t="inlineStr">
         <is>
           <t>2 vCPU | 4 GB RAM | 40 GB storage</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="4" t="inlineStr">
+      <c r="A14" s="3" t="inlineStr">
         <is>
           <t>Production / Browser Automation</t>
         </is>
       </c>
-      <c r="B14" s="4" t="inlineStr">
+      <c r="B14" s="3" t="inlineStr">
         <is>
           <t>4+ vCPU | 8-16 GB RAM | 80+ GB storage</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="6" t="inlineStr">
+      <c r="A15" s="2" t="inlineStr">
         <is>
           <t>— RESOURCE CONSUMPTION —</t>
         </is>
       </c>
-      <c r="B15" s="6" t="inlineStr"/>
+      <c r="B15" s="2" t="inlineStr"/>
     </row>
     <row r="16">
-      <c r="A16" s="4" t="inlineStr">
+      <c r="A16" s="3" t="inlineStr">
         <is>
           <t>Gateway Idle</t>
         </is>
       </c>
-      <c r="B16" s="4" t="inlineStr">
+      <c r="B16" s="3" t="inlineStr">
         <is>
           <t>Node.js Gateway idles at 300-500 MB RAM. CPU: 1-3%.</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="4" t="inlineStr">
+      <c r="A17" s="3" t="inlineStr">
         <is>
           <t>Browser Automation</t>
         </is>
       </c>
-      <c r="B17" s="4" t="inlineStr">
+      <c r="B17" s="3" t="inlineStr">
         <is>
           <t>8 GB RAM hard requirement. 3 browser nodes: 75-90% CPU.</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="4" t="inlineStr">
+      <c r="A18" s="3" t="inlineStr">
         <is>
           <t>Local LLM (8B model)</t>
         </is>
       </c>
-      <c r="B18" s="4" t="inlineStr">
+      <c r="B18" s="3" t="inlineStr">
         <is>
           <t>15-25% CPU | 2.8 GB peak RAM</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="4" t="inlineStr">
+      <c r="A19" s="3" t="inlineStr">
         <is>
           <t>Local LLM (14B model)</t>
         </is>
       </c>
-      <c r="B19" s="4" t="inlineStr">
+      <c r="B19" s="3" t="inlineStr">
         <is>
           <t>45-60% CPU | 5.4 GB peak RAM</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="6" t="inlineStr">
+      <c r="A20" s="2" t="inlineStr">
         <is>
           <t>— GPU REQUIREMENTS —</t>
         </is>
       </c>
-      <c r="B20" s="6" t="inlineStr"/>
+      <c r="B20" s="2" t="inlineStr"/>
     </row>
     <row r="21">
-      <c r="A21" s="4" t="inlineStr">
+      <c r="A21" s="3" t="inlineStr">
         <is>
           <t>Cloud LLM Mode</t>
         </is>
       </c>
-      <c r="B21" s="4" t="inlineStr">
+      <c r="B21" s="3" t="inlineStr">
         <is>
           <t>NO GPU required. OpenClaw acts as HTTP client to cloud APIs.</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="4" t="inlineStr">
+      <c r="A22" s="3" t="inlineStr">
         <is>
           <t>Local LLM Mode</t>
         </is>
       </c>
-      <c r="B22" s="4" t="inlineStr">
+      <c r="B22" s="3" t="inlineStr">
         <is>
           <t>GPU required. Rule of thumb: model params × 1GB VRAM (Q4 quantization).</t>
         </is>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="4" t="inlineStr">
+      <c r="A23" s="3" t="inlineStr">
         <is>
           <t>GPU Tiers</t>
         </is>
       </c>
-      <c r="B23" s="4" t="inlineStr">
+      <c r="B23" s="3" t="inlineStr">
         <is>
           <t>RTX 3060 (12GB) → 8B models | RTX 3090 (24GB) → 34B models | RTX 4090 (24GB) → 34-70B | A100 (40-80GB) → 70B+ | H100 (80GB) → 70-405B</t>
         </is>
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="4" t="inlineStr">
+      <c r="A24" s="3" t="inlineStr">
         <is>
           <t>Local LLM Stacks</t>
         </is>
       </c>
-      <c r="B24" s="4" t="inlineStr">
+      <c r="B24" s="3" t="inlineStr">
         <is>
           <t>Ollama, vLLM, TensorRT-LLM for GPU acceleration. LM Studio for CPU-only (limited).</t>
         </is>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="6" t="inlineStr">
+      <c r="A25" s="2" t="inlineStr">
         <is>
           <t>— COST BREAKDOWN —</t>
         </is>
       </c>
-      <c r="B25" s="6" t="inlineStr"/>
+      <c r="B25" s="2" t="inlineStr"/>
     </row>
     <row r="26">
-      <c r="A26" s="4" t="inlineStr">
+      <c r="A26" s="3" t="inlineStr">
         <is>
           <t>Budget Setup</t>
         </is>
       </c>
-      <c r="B26" s="4" t="inlineStr">
+      <c r="B26" s="3" t="inlineStr">
         <is>
           <t>$5-10/month total. Cheaper models (DeepSeek V3, Gemini Flash). Hetzner/Contabo VPS.</t>
         </is>
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="4" t="inlineStr">
+      <c r="A27" s="3" t="inlineStr">
         <is>
           <t>Standard Setup</t>
         </is>
       </c>
-      <c r="B27" s="4" t="inlineStr">
+      <c r="B27" s="3" t="inlineStr">
         <is>
           <t>$15-30/month. Claude Sonnet 4 or GPT-4o. 4 GB RAM VPS.</t>
         </is>
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="4" t="inlineStr">
+      <c r="A28" s="3" t="inlineStr">
         <is>
           <t>Heavy Use</t>
         </is>
       </c>
-      <c r="B28" s="4" t="inlineStr">
+      <c r="B28" s="3" t="inlineStr">
         <is>
           <t>$62-224+/month. Browser automation + expensive models.</t>
         </is>
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="4" t="inlineStr">
+      <c r="A29" s="3" t="inlineStr">
         <is>
           <t>Enterprise (100 people)</t>
         </is>
       </c>
-      <c r="B29" s="4" t="inlineStr">
+      <c r="B29" s="3" t="inlineStr">
         <is>
           <t>$30,000-50,000/month (per-person model with Claude Opus).</t>
         </is>
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="4" t="inlineStr">
+      <c r="A30" s="3" t="inlineStr">
         <is>
           <t>Hidden Costs</t>
         </is>
       </c>
-      <c r="B30" s="4" t="inlineStr">
+      <c r="B30" s="3" t="inlineStr">
         <is>
           <t>System prompt token burn: $5-30/mo | Heartbeat checks: $0-90/mo | Maintenance: 2-5 hrs/mo</t>
         </is>
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="4" t="inlineStr">
+      <c r="A31" s="3" t="inlineStr">
         <is>
           <t>Free Option</t>
         </is>
       </c>
-      <c r="B31" s="4" t="inlineStr">
+      <c r="B31" s="3" t="inlineStr">
         <is>
           <t>Oracle Cloud Always Free tier (24 GB RAM).</t>
         </is>
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="6" t="inlineStr">
+      <c r="A32" s="2" t="inlineStr">
         <is>
           <t>— KEY DISTINCTION —</t>
         </is>
       </c>
-      <c r="B32" s="6" t="inlineStr"/>
+      <c r="B32" s="2" t="inlineStr"/>
     </row>
     <row r="33">
-      <c r="A33" s="4" t="inlineStr">
+      <c r="A33" s="3" t="inlineStr">
         <is>
           <t>Not a Coding Agent</t>
         </is>
       </c>
-      <c r="B33" s="4" t="inlineStr">
+      <c r="B33" s="3" t="inlineStr">
         <is>
           <t>OpenClaw is a general-purpose personal assistant, NOT a coding agent like Devin or Claude Code. It automates tasks like email, calendar, smart home, and workflows across messaging platforms.</t>
         </is>

</xml_diff>

<commit_message>
Add NVIDIA GTC 2026 OpenClaw/NemoClaw data
New 'NVIDIA GTC – OpenClaw' tab covering:
- Jensen Huang keynote: OpenClaw as 'the OS for personal AI'
- NemoClaw enterprise stack (OpenClaw + Nemotron + OpenShell)
- OpenShell security runtime (Landlock, seccomp, policy guardrails)
- Nemotron model family (Super 120B, Nano 4B, Ultra 253B, Super 49B)
- PinchBench leaderboard (Nemotron 85.6% vs Claude 86.9%)
- Hardware platforms (DGX Spark, DGX Station, RTX PCs)
- Enterprise partners (Adobe, Salesforce, SAP, ServiceNow, etc.)
- Cost impact (Vera Rubin 40% lower cost-per-token, Nemotron >50% savings)
- Adoption data (250K stars, 2.2M npm downloads, 65% enterprise users)

Also updated OpenClaw Deep Dive tab with GTC 2026 validation section.

Co-authored-by: ms4674 <ms4674@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/OpenClaw_Architecture_Comparison.xlsx
+++ b/OpenClaw_Architecture_Comparison.xlsx
@@ -9,10 +9,11 @@
   <sheets>
     <sheet name="OpenClaw vs Claude Cowork" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Architecture Comparison" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Compute Requirements" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Pricing Comparison" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Strategic Notes" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="OpenClaw Deep Dive" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="NVIDIA GTC – OpenClaw" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Compute Requirements" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Pricing Comparison" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Strategic Notes" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="OpenClaw Deep Dive" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -51,7 +52,7 @@
       <sz val="10"/>
     </font>
   </fonts>
-  <fills count="8">
+  <fills count="9">
     <fill>
       <patternFill/>
     </fill>
@@ -94,6 +95,12 @@
         <bgColor rgb="00FCE4D6"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="0076B900"/>
+        <bgColor rgb="0076B900"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -113,7 +120,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
@@ -138,6 +145,9 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -2541,6 +2551,495 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:B35"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="32" customWidth="1" min="1" max="1"/>
+    <col width="110" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="9" t="inlineStr">
+        <is>
+          <t>Topic</t>
+        </is>
+      </c>
+      <c r="B1" s="9" t="inlineStr">
+        <is>
+          <t>Details</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>— JENSEN HUANG KEYNOTE HIGHLIGHTS —</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>Strategic Positioning</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Jensen Huang declared: "Every single company in the world today has to have an OpenClaw strategy."
+Positioned OpenClaw as "the operating system for personal AI" — comparable to Windows, Linux, and HTML.
+NVIDIA views OpenClaw as a foundational layer for the emerging AI agent ecosystem.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>Adoption Trajectory</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>OpenClaw surpassed Linux's adoption curve — reaching equivalent milestones in 3 weeks vs. Linux's 30-year trajectory.
+250,000+ GitHub stars in 60 days (surpassing React's 10-year record).
+2.2 million weekly npm downloads.
+Described by Huang as "the most popular open source project in the history of humanity."</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>Enterprise Penetration</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>65% of OpenClaw users are in enterprise sectors.
+Gartner projects 40% of enterprise applications will embed task-specific AI agents by end of 2026 (up from &lt;5% in 2025).
+Global agentic AI market: $7.6B (2025) → projected $199B by 2034.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>— NEMOCLAW: NVIDIA'S OPENCLAW STACK —</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="3" t="inlineStr">
+        <is>
+          <t>What Is NemoClaw</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t>An enterprise-grade, open-source (Apache 2.0) software stack that layers security, privacy, and runtime controls on top of OpenClaw.
+Pre-packaged: OpenClaw + NVIDIA Nemotron models + NVIDIA OpenShell runtime — installable with a single command.
+Enables production-ready agent deployment in under 1 hour.
+GitHub: github.com/NVIDIA/NemoClaw (alpha status as of March 2026).</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="3" t="inlineStr">
+        <is>
+          <t>NemoClaw Components</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="inlineStr">
+        <is>
+          <t>1. OpenClaw: Core AI agent framework (task execution, messaging, MCP skills).
+2. NVIDIA OpenShell: Secure sandboxed runtime with kernel-level isolation (Landlock LSM, seccomp, bubblewrap).
+3. Nemotron Models: Open models optimized for agentic workloads (see below).
+4. Inference Routing: Intercepts all model calls to enforce privacy &amp; cost constraints. Supports local vLLM, NIM, or NVIDIA cloud.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="3" t="inlineStr">
+        <is>
+          <t>NemoClaw Inference Profiles</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t>Three profiles available:
+• default: NVIDIA cloud via integrate.api.nvidia.com (Nemotron-3-Super-120B)
+• nim-local: Local NVIDIA NIM service deployment
+• vllm: Local vLLM development option
+All profiles support policy-based cost and privacy constraints.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>— NVIDIA OPENSHELL SECURITY RUNTIME —</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="3" t="inlineStr">
+        <is>
+          <t>Architecture</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="inlineStr">
+        <is>
+          <t>Open-sourced March 2026 under Apache 2.0.
+Provides sandboxed execution between AI agents and the host OS.
+Agents (OpenClaw, Claude Code, Codex) run unmodified inside OpenShell — zero code changes required.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="3" t="inlineStr">
+        <is>
+          <t>Static Policies
+(locked at sandbox creation)</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="inlineStr">
+        <is>
+          <t>• Filesystem: Read-only / read-write directory lists enforced via Landlock LSM kernel-level isolation.
+• Process: Agent runs as unprivileged user (defaults to 'sandbox'); rejects root. Seccomp filters block dangerous syscalls.
+• Landlock compatibility modes: 'best_effort' or 'hard_requirement'.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="3" t="inlineStr">
+        <is>
+          <t>Dynamic Policies
+(hot-reloadable at runtime)</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>• Network: Per-binary control (which executables can reach which endpoints). Protocol inspection for REST with TLS termination.
+• Per-method control: Governs specific API calls or shell functions.
+• Per-endpoint control: Limits traffic to specific IPs/domains.
+• Per-binary control: Restricts which executables (git, curl, python) agents can invoke.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="3" t="inlineStr">
+        <is>
+          <t>Audit &amp; Compliance</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="inlineStr">
+        <is>
+          <t>All agent actions logged in audit trails for compliance and debugging.
+Developed in response to documented OpenClaw vulnerabilities (indirect prompt injection, malicious payloads in customization hub).
+Declarative YAML policy configuration.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>— NEMOTRON MODEL FAMILY FOR OPENCLAW —</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="3" t="inlineStr">
+        <is>
+          <t>Nemotron 3 Super 120B</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="inlineStr">
+        <is>
+          <t>Parameters: 120B total, only 12B active (MoE architecture).
+Architecture: Hybrid Mamba-Transformer Mixture-of-Experts.
+Context Window: 1M tokens native.
+PinchBench Score: 85.6% (top open model; competitive with Claude Sonnet 4.6 at 86.9%).
+Throughput: 5× higher than predecessor; 42,855 tok/s prompt processing on DGX Spark.
+Generation: 18 tok/s on DGX Spark (128K input tokens).
+End-to-end latency: 99.4s for 128K token input on DGX Spark.
+License: Fully open (weights, datasets, recipes).</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="3" t="inlineStr">
+        <is>
+          <t>Nemotron 3 Nano 4B</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="inlineStr">
+        <is>
+          <t>Parameters: 4B.
+Target: Resource-constrained RTX AI PCs, games, and apps.
+Strong instruction-following and tool use with minimal VRAM.
+Context Window: 131,072 tokens.
+Designed for local agents on consumer hardware.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="3" t="inlineStr">
+        <is>
+          <t>Nemotron Ultra 253B</t>
+        </is>
+      </c>
+      <c r="B18" s="3" t="inlineStr">
+        <is>
+          <t>Parameters: 253B.
+Context Window: 131,072 tokens; 4,096 max output.
+For enterprise-grade deep reasoning and complex multi-agent tasks.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="3" t="inlineStr">
+        <is>
+          <t>Nemotron Super 49B v1.5</t>
+        </is>
+      </c>
+      <c r="B19" s="3" t="inlineStr">
+        <is>
+          <t>Parameters: 49B.
+Context Window: 131,072 tokens; 4,096 max output.
+Mid-tier option balancing performance and resource needs.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>— PINCHBENCH: OPENCLAW AGENT BENCHMARK —</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="3" t="inlineStr">
+        <is>
+          <t>What Is PinchBench</t>
+        </is>
+      </c>
+      <c r="B21" s="3" t="inlineStr">
+        <is>
+          <t>The first benchmarking system specifically designed for OpenClaw agents.
+23 tasks across 8 categories: long-term memory retrieval, inbox triage, spreadsheet processing, scheduling, and more.
+Tests real-world agentic task completion, not just code generation.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="3" t="inlineStr">
+        <is>
+          <t>Leaderboard
+(Success Rate, 2026)</t>
+        </is>
+      </c>
+      <c r="B22" s="3" t="inlineStr">
+        <is>
+          <t>1. Claude Sonnet 4.6:           86.9%
+2. GPT-5.4:                     86.4%
+3. Claude Opus 4.6:             86.3%
+4. Nemotron-3-Super-120B:       85.6%  ← Top open model
+5. Claude Opus 4.5:             85.4%
+(Gemini 3 Flash Preview reported at 95.1% in earlier runs)</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="3" t="inlineStr">
+        <is>
+          <t>Key Insight</t>
+        </is>
+      </c>
+      <c r="B23" s="3" t="inlineStr">
+        <is>
+          <t>NVIDIA's open Nemotron-3-Super-120B trails the best proprietary model (Claude Sonnet 4.6) by only 1.3 percentage points.
+This near-parity enables fully local, private OpenClaw deployments without significant quality loss.
+Cost: $0 ongoing API fees vs. $5-420/mo for cloud models.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>— NVIDIA HARDWARE FOR OPENCLAW —</t>
+        </is>
+      </c>
+      <c r="B24" s="2" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="3" t="inlineStr">
+        <is>
+          <t>DGX Spark
+(Desktop AI Supercomputer)</t>
+        </is>
+      </c>
+      <c r="B25" s="3" t="inlineStr">
+        <is>
+          <t>GPU: NVIDIA Blackwell (5th gen Tensor Cores, 4th gen RT Cores).
+CPU: 20-core Arm (10× Cortex-X925 + 10× Cortex-A725).
+Memory: 128 GB LPDDR5x unified (273 GB/s bandwidth).
+Storage: 1 TB or 4 TB NVMe M.2.
+AI Compute: Up to 1,000 TOPS; 1 PFLOP at FP4 with sparsity.
+CUDA Cores: 6,144.
+Form Factor: 150mm × 150mm × 50.5mm, 1.2 kg.
+Power: 240W external (140W GPU TDP).
+Model Support: Up to 200B parameters (405B in dual-Spark config).
+Concurrency: 4 simultaneous subagents with ~3× throughput increase at 2.6× time.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="3" t="inlineStr">
+        <is>
+          <t>DGX Station
+(Enterprise AI Supercomputer)</t>
+        </is>
+      </c>
+      <c r="B26" s="3" t="inlineStr">
+        <is>
+          <t>GB300 variant: 748 GB coherent memory.
+Targets enterprise multi-agent workloads.
+Supports the full Nemotron model family including Ultra 253B.
+Designed for always-on, server-class OpenClaw deployments.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="3" t="inlineStr">
+        <is>
+          <t>RTX PRO Workstations
+&amp; GeForce RTX PCs</t>
+        </is>
+      </c>
+      <c r="B27" s="3" t="inlineStr">
+        <is>
+          <t>Nemotron 3 Nano 4B runs on consumer RTX hardware.
+Dell Pro Max systems with GB10 (128 GB unified memory) available.
+Entry point for local OpenClaw agents without enterprise hardware.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="inlineStr">
+        <is>
+          <t>— ENTERPRISE PARTNERS (AGENT TOOLKIT) —</t>
+        </is>
+      </c>
+      <c r="B28" s="2" t="inlineStr"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="3" t="inlineStr">
+        <is>
+          <t>Tier-1 Partners</t>
+        </is>
+      </c>
+      <c r="B29" s="3" t="inlineStr">
+        <is>
+          <t>Adobe, Salesforce, SAP, ServiceNow, Siemens, CrowdStrike, Atlassian, Palantir.
+All building with the NVIDIA Agent Toolkit which includes NemoClaw.
+Focus: secure, enterprise-grade agentic AI deployments.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="inlineStr">
+        <is>
+          <t>— COST IMPACT —</t>
+        </is>
+      </c>
+      <c r="B30" s="2" t="inlineStr"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="3" t="inlineStr">
+        <is>
+          <t>Vera Rubin Platform</t>
+        </is>
+      </c>
+      <c r="B31" s="3" t="inlineStr">
+        <is>
+          <t>NVIDIA's next-gen inference platform delivers 40% lower cost-per-token vs. Blackwell deployments.
+Directly reduces OpenClaw operational costs for cloud-inference users.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="3" t="inlineStr">
+        <is>
+          <t>Nemotron Cost Advantage</t>
+        </is>
+      </c>
+      <c r="B32" s="3" t="inlineStr">
+        <is>
+          <t>Nemotron models reduce query costs by &gt;50% vs. comparable proprietary models (per NVIDIA).
+Local inference: $0 ongoing API costs (hardware amortization only).
+Cloud Nemotron via NVIDIA API: significantly cheaper than Claude/GPT equivalents.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="3" t="inlineStr">
+        <is>
+          <t>TCO Comparison:
+Local NemoClaw on DGX Spark
+vs. Cloud OpenClaw</t>
+        </is>
+      </c>
+      <c r="B33" s="3" t="inlineStr">
+        <is>
+          <t>Cloud OpenClaw (Claude Opus): $300-500/mo per agent in API fees.
+Local NemoClaw (DGX Spark): Hardware one-time cost; $0/mo API fees.
+Break-even: DGX Spark investment pays back in months for heavy users.
+Quality gap: Only 1.3% PinchBench difference (85.6% vs. 86.9%).</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="2" t="inlineStr">
+        <is>
+          <t>— SUMMARY: GTC 2026 SIGNIFICANCE FOR OPENCLAW —</t>
+        </is>
+      </c>
+      <c r="B34" s="2" t="inlineStr"/>
+    </row>
+    <row r="35">
+      <c r="A35" s="3" t="inlineStr">
+        <is>
+          <t>Strategic Takeaway</t>
+        </is>
+      </c>
+      <c r="B35" s="3" t="inlineStr">
+        <is>
+          <t>NVIDIA's GTC 2026 announcements fundamentally elevate OpenClaw from a community project to an enterprise-grade platform:
+1. VALIDATION: Jensen Huang positioning OpenClaw as essential as Windows/Linux legitimizes it for enterprise.
+2. SECURITY: OpenShell/NemoClaw solves the #1 enterprise blocker (security concerns) with kernel-level sandboxing.
+3. LOCAL INFERENCE: Nemotron 3 Super 120B achieves near-parity with Claude/GPT at zero API cost.
+4. HARDWARE ECOSYSTEM: DGX Spark ($3K-$5K est.) to DGX Station creates a clear hardware upgrade path.
+5. ENTERPRISE PARTNERS: Adobe, Salesforce, SAP, ServiceNow adoption signals mainstream enterprise readiness.
+6. COST REDUCTION: Vera Rubin platform + Nemotron models compress costs by 40-50%+.
+Net effect: OpenClaw is now positioned as the default AI agent runtime with NVIDIA's full-stack backing, comparable to how Linux became the default server OS with Red Hat/IBM enterprise support.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:F17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -3079,7 +3578,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -3709,7 +4208,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -4267,13 +4766,13 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B33"/>
+  <dimension ref="A1:B40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -4631,7 +5130,7 @@
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>— KEY DISTINCTION —</t>
+          <t>— NVIDIA GTC 2026 VALIDATION —</t>
         </is>
       </c>
       <c r="B32" s="2" t="inlineStr"/>
@@ -4639,10 +5138,90 @@
     <row r="33">
       <c r="A33" s="3" t="inlineStr">
         <is>
+          <t>NVIDIA Partnership</t>
+        </is>
+      </c>
+      <c r="B33" s="3" t="inlineStr">
+        <is>
+          <t>Jensen Huang (GTC 2026): "Every single company in the world today has to have an OpenClaw strategy." Positioned as "the operating system for personal AI."</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="3" t="inlineStr">
+        <is>
+          <t>NemoClaw Stack</t>
+        </is>
+      </c>
+      <c r="B34" s="3" t="inlineStr">
+        <is>
+          <t>NVIDIA's enterprise wrapper: OpenClaw + Nemotron models + OpenShell sandboxed runtime. Apache 2.0 license. Single-command install. Production-ready in &lt;1 hour.</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="3" t="inlineStr">
+        <is>
+          <t>Nemotron 3 Super 120B</t>
+        </is>
+      </c>
+      <c r="B35" s="3" t="inlineStr">
+        <is>
+          <t>Top open model on PinchBench (85.6%), only 1.3% behind Claude Sonnet 4.6 (86.9%). 12B active params (MoE). 1M token context. 42,855 tok/s on DGX Spark.</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="3" t="inlineStr">
+        <is>
+          <t>Hardware Ecosystem</t>
+        </is>
+      </c>
+      <c r="B36" s="3" t="inlineStr">
+        <is>
+          <t>DGX Spark (128 GB, 1 PFLOP, desktop form) → DGX Station (748 GB, enterprise) → RTX PCs (Nemotron Nano 4B). Full upgrade path for local OpenClaw inference.</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="3" t="inlineStr">
+        <is>
+          <t>Enterprise Partners</t>
+        </is>
+      </c>
+      <c r="B37" s="3" t="inlineStr">
+        <is>
+          <t>Adobe, Salesforce, SAP, ServiceNow, Siemens, CrowdStrike, Atlassian, Palantir — all building with NVIDIA Agent Toolkit / NemoClaw.</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="3" t="inlineStr">
+        <is>
+          <t>Adoption (GTC Data)</t>
+        </is>
+      </c>
+      <c r="B38" s="3" t="inlineStr">
+        <is>
+          <t>250K+ GitHub stars in 60 days. 2.2M weekly npm downloads. 65% of users in enterprise sectors. Surpassed Linux adoption speed (3 weeks vs. 30 years).</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="2" t="inlineStr">
+        <is>
+          <t>— KEY DISTINCTION —</t>
+        </is>
+      </c>
+      <c r="B39" s="2" t="inlineStr"/>
+    </row>
+    <row r="40">
+      <c r="A40" s="3" t="inlineStr">
+        <is>
           <t>Not a Coding Agent</t>
         </is>
       </c>
-      <c r="B33" s="3" t="inlineStr">
+      <c r="B40" s="3" t="inlineStr">
         <is>
           <t>OpenClaw is a general-purpose personal assistant, NOT a coding agent like Devin or Claude Code. It automates tasks like email, calendar, smart home, and workflows across messaging platforms.</t>
         </is>

</xml_diff>